<commit_message>
Complete all 166 Audius links using both profiles and verified source durations
</commit_message>
<xml_diff>
--- a/Ch-D_music_catalog.xlsx
+++ b/Ch-D_music_catalog.xlsx
@@ -137,13 +137,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>102</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7">
@@ -884,8 +884,12 @@
       <c r="H6" s="9" t="inlineStr"/>
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="11" t="n">
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/40k-steps-to-heresy-моделист</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="n">
         <v>0.00325</v>
       </c>
       <c r="M6" s="10" t="inlineStr">
@@ -924,8 +928,12 @@
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
-      <c r="L7" s="11" t="n">
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/_ddn-котлетка</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="n">
         <v>0.001875578703703704</v>
       </c>
       <c r="M7" s="10" t="inlineStr">
@@ -964,8 +972,12 @@
       <c r="H8" s="9" t="inlineStr"/>
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="11" t="n">
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/agonit-rivendare</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="n">
         <v>0.001414930555555556</v>
       </c>
       <c r="M8" s="10" t="inlineStr">
@@ -1004,8 +1016,12 @@
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
-      <c r="L9" s="11" t="n">
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/baskova-зелёный-слоник-concert-version</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M9" s="10" t="inlineStr">
@@ -1044,11 +1060,15 @@
       <c r="H10" s="9" t="inlineStr"/>
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
-      <c r="L10" s="11" t="n">
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/black-hand-lament-1</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="n">
         <v>0.001909722222222222</v>
       </c>
-      <c r="M10" s="12" t="inlineStr">
+      <c r="M10" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -1080,9 +1100,13 @@
       <c r="H11" s="9" t="inlineStr"/>
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
-      <c r="L11" s="11" t="n">
-        <v>0.002170486111111111</v>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/bring-me-the-execute-прокачка</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>0.002115595868055555</v>
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
@@ -1116,8 +1140,12 @@
       <c r="H12" s="9" t="inlineStr"/>
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
-      <c r="L12" s="11" t="n">
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/broken-shards-of-dark-talent</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="n">
         <v>0.001448842592592593</v>
       </c>
       <c r="M12" s="10" t="inlineStr">
@@ -1164,11 +1192,15 @@
       <c r="H13" s="9" t="inlineStr"/>
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
-      <c r="L13" s="11" t="n">
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/bronzebeard-генни</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="n">
         <v>0.003032754629629629</v>
       </c>
-      <c r="M13" s="12" t="inlineStr">
+      <c r="M13" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -1212,11 +1244,15 @@
       <c r="H14" s="9" t="inlineStr"/>
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="9" t="inlineStr"/>
-      <c r="K14" s="9" t="inlineStr"/>
-      <c r="L14" s="11" t="n">
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/bronzebeard-чорная-гора</t>
+        </is>
+      </c>
+      <c r="L14" s="12" t="n">
         <v>0.002198842592592593</v>
       </c>
-      <c r="M14" s="12" t="inlineStr">
+      <c r="M14" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -1256,11 +1292,15 @@
       <c r="H15" s="9" t="inlineStr"/>
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="9" t="inlineStr"/>
-      <c r="L15" s="11" t="n">
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/chd-bustaz-греем-до-утра</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="n">
         <v>0.002356944444444444</v>
       </c>
-      <c r="M15" s="12" t="inlineStr">
+      <c r="M15" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -1292,12 +1332,12 @@
       <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr"/>
-      <c r="K16" s="13" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/cript-cover-den-1</t>
         </is>
       </c>
-      <c r="L16" s="11" t="n">
+      <c r="L16" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M16" s="10" t="inlineStr">
@@ -1332,12 +1372,12 @@
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="9" t="inlineStr"/>
-      <c r="K17" s="13" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/cryptonit-–-проклятие-крипты</t>
         </is>
       </c>
-      <c r="L17" s="11" t="n">
+      <c r="L17" s="12" t="n">
         <v>0.002508101851851852</v>
       </c>
       <c r="M17" s="10" t="inlineStr">
@@ -1372,12 +1412,12 @@
       <c r="H18" s="9" t="inlineStr"/>
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="9" t="inlineStr"/>
-      <c r="K18" s="13" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/digital-fury</t>
         </is>
       </c>
-      <c r="L18" s="11" t="n">
+      <c r="L18" s="12" t="n">
         <v>0.002633217592592592</v>
       </c>
       <c r="M18" s="10" t="inlineStr">
@@ -1420,15 +1460,15 @@
       <c r="H19" s="9" t="inlineStr"/>
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="9" t="inlineStr"/>
-      <c r="K19" s="13" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/dominus-agonetti-rivendare</t>
         </is>
       </c>
-      <c r="L19" s="11" t="n">
+      <c r="L19" s="12" t="n">
         <v>0.003843055555555556</v>
       </c>
-      <c r="M19" s="12" t="inlineStr">
+      <c r="M19" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -1468,12 +1508,12 @@
       <c r="H20" s="9" t="inlineStr"/>
       <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="9" t="inlineStr"/>
-      <c r="K20" s="13" t="inlineStr">
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
         </is>
       </c>
-      <c r="L20" s="11" t="n">
+      <c r="L20" s="12" t="n">
         <v>0.003261921296296296</v>
       </c>
       <c r="M20" s="10" t="inlineStr">
@@ -1516,15 +1556,15 @@
       <c r="H21" s="9" t="inlineStr"/>
       <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="9" t="inlineStr"/>
-      <c r="K21" s="13" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-ii-duetus-in-ruinis-stratholmi-aria-rivendari-et-isidis</t>
         </is>
       </c>
-      <c r="L21" s="11" t="n">
+      <c r="L21" s="12" t="n">
         <v>0.003152777777777777</v>
       </c>
-      <c r="M21" s="12" t="inlineStr">
+      <c r="M21" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -1560,12 +1600,12 @@
       <c r="H22" s="9" t="inlineStr"/>
       <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="9" t="inlineStr"/>
-      <c r="K22" s="13" t="inlineStr">
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/edovuaruhaindo-fujōnaru-te-no-kayō</t>
         </is>
       </c>
-      <c r="L22" s="11" t="n">
+      <c r="L22" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M22" s="10" t="inlineStr">
@@ -1608,12 +1648,12 @@
       <c r="H23" s="9" t="inlineStr"/>
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="9" t="inlineStr"/>
-      <c r="K23" s="13" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/fakmod-sirus</t>
         </is>
       </c>
-      <c r="L23" s="11" t="n">
+      <c r="L23" s="12" t="n">
         <v>0.001800810185185185</v>
       </c>
       <c r="M23" s="10" t="inlineStr">
@@ -1652,12 +1692,12 @@
       <c r="H24" s="9" t="inlineStr"/>
       <c r="I24" s="10" t="inlineStr"/>
       <c r="J24" s="9" t="inlineStr"/>
-      <c r="K24" s="13" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/fordring-о-король</t>
         </is>
       </c>
-      <c r="L24" s="11" t="n">
+      <c r="L24" s="12" t="n">
         <v>0.001606134259259259</v>
       </c>
       <c r="M24" s="10" t="inlineStr">
@@ -1700,12 +1740,12 @@
       <c r="H25" s="9" t="inlineStr"/>
       <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="9" t="inlineStr"/>
-      <c r="K25" s="13" t="inlineStr">
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/fuckmode-wow-sirus</t>
         </is>
       </c>
-      <c r="L25" s="11" t="n">
+      <c r="L25" s="12" t="n">
         <v>0.001800578703703704</v>
       </c>
       <c r="M25" s="10" t="inlineStr">
@@ -1748,12 +1788,12 @@
       <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="10" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
-      <c r="K26" s="13" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/greywick-hill-мэрри-хоуп</t>
         </is>
       </c>
-      <c r="L26" s="11" t="n">
+      <c r="L26" s="12" t="n">
         <v>0.00335150462962963</v>
       </c>
       <c r="M26" s="10" t="inlineStr">
@@ -1792,15 +1832,15 @@
       <c r="H27" s="9" t="inlineStr"/>
       <c r="I27" s="10" t="inlineStr"/>
       <c r="J27" s="9" t="inlineStr"/>
-      <c r="K27" s="13" t="inlineStr">
+      <c r="K27" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/hastwood-владыка-черного-алмаза</t>
         </is>
       </c>
-      <c r="L27" s="11" t="n">
+      <c r="L27" s="12" t="n">
         <v>0.002384953703703704</v>
       </c>
-      <c r="M27" s="12" t="inlineStr">
+      <c r="M27" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -1836,12 +1876,12 @@
       <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="9" t="inlineStr"/>
-      <c r="K28" s="13" t="inlineStr">
+      <c r="K28" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/hastwood-ужас-в-вандермаре</t>
         </is>
       </c>
-      <c r="L28" s="11" t="n">
+      <c r="L28" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M28" s="10" t="inlineStr">
@@ -1876,12 +1916,12 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="10" t="inlineStr"/>
       <c r="J29" s="9" t="inlineStr"/>
-      <c r="K29" s="13" t="inlineStr">
+      <c r="K29" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/heilung_-_traust_skysoundcc</t>
         </is>
       </c>
-      <c r="L29" s="11" t="n">
+      <c r="L29" s="12" t="n">
         <v>0.006855324074074074</v>
       </c>
       <c r="M29" s="10" t="inlineStr">
@@ -1920,12 +1960,12 @@
       <c r="H30" s="9" t="inlineStr"/>
       <c r="I30" s="10" t="inlineStr"/>
       <c r="J30" s="9" t="inlineStr"/>
-      <c r="K30" s="13" t="inlineStr">
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/hestia-discordiam-sugere</t>
         </is>
       </c>
-      <c r="L30" s="11" t="n">
+      <c r="L30" s="12" t="n">
         <v>0.001683912037037037</v>
       </c>
       <c r="M30" s="10" t="inlineStr">
@@ -1968,12 +2008,12 @@
       <c r="H31" s="9" t="inlineStr"/>
       <c r="I31" s="10" t="inlineStr"/>
       <c r="J31" s="9" t="inlineStr"/>
-      <c r="K31" s="13" t="inlineStr">
+      <c r="K31" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/homabrut-три-ночи</t>
         </is>
       </c>
-      <c r="L31" s="11" t="n">
+      <c r="L31" s="12" t="n">
         <v>0.003156134259259259</v>
       </c>
       <c r="M31" s="10" t="inlineStr">
@@ -2016,15 +2056,15 @@
       <c r="H32" s="9" t="inlineStr"/>
       <c r="I32" s="10" t="inlineStr"/>
       <c r="J32" s="9" t="inlineStr"/>
-      <c r="K32" s="13" t="inlineStr">
+      <c r="K32" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/kanye-brown-прогрелись-в-котле</t>
         </is>
       </c>
-      <c r="L32" s="11" t="n">
+      <c r="L32" s="12" t="n">
         <v>0.003093055555555555</v>
       </c>
-      <c r="M32" s="12" t="inlineStr">
+      <c r="M32" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -2060,12 +2100,12 @@
       <c r="H33" s="9" t="inlineStr"/>
       <c r="I33" s="10" t="inlineStr"/>
       <c r="J33" s="9" t="inlineStr"/>
-      <c r="K33" s="13" t="inlineStr">
+      <c r="K33" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/kushnerit-cursed-crypt</t>
         </is>
       </c>
-      <c r="L33" s="11" t="n">
+      <c r="L33" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M33" s="10" t="inlineStr">
@@ -2104,12 +2144,12 @@
       <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="10" t="inlineStr"/>
       <c r="J34" s="9" t="inlineStr"/>
-      <c r="K34" s="13" t="inlineStr">
+      <c r="K34" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/lightfair-мор-ладим</t>
         </is>
       </c>
-      <c r="L34" s="11" t="n">
+      <c r="L34" s="12" t="n">
         <v>0.002145023148148149</v>
       </c>
       <c r="M34" s="10" t="inlineStr">
@@ -2152,12 +2192,12 @@
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="10" t="inlineStr"/>
       <c r="J35" s="9" t="inlineStr"/>
-      <c r="K35" s="13" t="inlineStr">
+      <c r="K35" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/morgenshtern-x-chd-саркофаг</t>
         </is>
       </c>
-      <c r="L35" s="11" t="n">
+      <c r="L35" s="12" t="n">
         <v>0.002070023148148148</v>
       </c>
       <c r="M35" s="10" t="inlineStr">
@@ -2196,12 +2236,12 @@
       <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="10" t="inlineStr"/>
       <c r="J36" s="9" t="inlineStr"/>
-      <c r="K36" s="13" t="inlineStr">
+      <c r="K36" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/mrcrow-блю-юр</t>
         </is>
       </c>
-      <c r="L36" s="11" t="n">
+      <c r="L36" s="12" t="n">
         <v>0.002141898148148148</v>
       </c>
       <c r="M36" s="10" t="inlineStr">
@@ -2252,15 +2292,15 @@
       <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="10" t="inlineStr"/>
       <c r="J37" s="9" t="inlineStr"/>
-      <c r="K37" s="13" t="inlineStr">
+      <c r="K37" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/nagvar-жизнь-хороша</t>
         </is>
       </c>
-      <c r="L37" s="11" t="n">
+      <c r="L37" s="12" t="n">
         <v>0.002015277777777778</v>
       </c>
-      <c r="M37" s="12" t="inlineStr">
+      <c r="M37" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -2300,15 +2340,15 @@
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="10" t="inlineStr"/>
       <c r="J38" s="9" t="inlineStr"/>
-      <c r="K38" s="13" t="inlineStr">
+      <c r="K38" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/nasramka-за-калич-да</t>
         </is>
       </c>
-      <c r="L38" s="11" t="n">
+      <c r="L38" s="12" t="n">
         <v>0.001210532407407407</v>
       </c>
-      <c r="M38" s="12" t="inlineStr">
+      <c r="M38" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -2340,12 +2380,12 @@
       <c r="H39" s="9" t="inlineStr"/>
       <c r="I39" s="10" t="inlineStr"/>
       <c r="J39" s="9" t="inlineStr"/>
-      <c r="K39" s="13" t="inlineStr">
+      <c r="K39" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
         </is>
       </c>
-      <c r="L39" s="11" t="n">
+      <c r="L39" s="12" t="n">
         <v>0.001571064814814815</v>
       </c>
       <c r="M39" s="10" t="inlineStr">
@@ -2384,12 +2424,12 @@
       <c r="H40" s="9" t="inlineStr"/>
       <c r="I40" s="10" t="inlineStr"/>
       <c r="J40" s="9" t="inlineStr"/>
-      <c r="K40" s="13" t="inlineStr">
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neoromant-о-король</t>
         </is>
       </c>
-      <c r="L40" s="11" t="n">
+      <c r="L40" s="12" t="n">
         <v>0.001606134259259259</v>
       </c>
       <c r="M40" s="10" t="inlineStr">
@@ -2428,15 +2468,15 @@
       <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="10" t="inlineStr"/>
       <c r="J41" s="9" t="inlineStr"/>
-      <c r="K41" s="13" t="inlineStr">
+      <c r="K41" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-singularity</t>
         </is>
       </c>
-      <c r="L41" s="11" t="n">
+      <c r="L41" s="12" t="n">
         <v>0.002292476851851852</v>
       </c>
-      <c r="M41" s="12" t="inlineStr">
+      <c r="M41" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -2472,12 +2512,12 @@
       <c r="H42" s="9" t="inlineStr"/>
       <c r="I42" s="10" t="inlineStr"/>
       <c r="J42" s="9" t="inlineStr"/>
-      <c r="K42" s="13" t="inlineStr">
+      <c r="K42" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-agonito-no-kokoro</t>
         </is>
       </c>
-      <c r="L42" s="11" t="n">
+      <c r="L42" s="12" t="n">
         <v>0.00226724537037037</v>
       </c>
       <c r="M42" s="10" t="inlineStr">
@@ -2516,12 +2556,12 @@
       <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="10" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr"/>
-      <c r="K43" s="13" t="inlineStr">
+      <c r="K43" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-crypt</t>
         </is>
       </c>
-      <c r="L43" s="11" t="n">
+      <c r="L43" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M43" s="10" t="inlineStr">
@@ -2560,12 +2600,12 @@
       <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="10" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr"/>
-      <c r="K44" s="13" t="inlineStr">
+      <c r="K44" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-destiny</t>
         </is>
       </c>
-      <c r="L44" s="11" t="n">
+      <c r="L44" s="12" t="n">
         <v>0.001761342592592593</v>
       </c>
       <c r="M44" s="10" t="inlineStr">
@@ -2608,12 +2648,12 @@
       <c r="H45" s="9" t="inlineStr"/>
       <c r="I45" s="10" t="inlineStr"/>
       <c r="J45" s="9" t="inlineStr"/>
-      <c r="K45" s="13" t="inlineStr">
+      <c r="K45" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
         </is>
       </c>
-      <c r="L45" s="11" t="n">
+      <c r="L45" s="12" t="n">
         <v>0.002830324074074074</v>
       </c>
       <c r="M45" s="10" t="inlineStr">
@@ -2652,12 +2692,12 @@
       <c r="H46" s="9" t="inlineStr"/>
       <c r="I46" s="10" t="inlineStr"/>
       <c r="J46" s="9" t="inlineStr"/>
-      <c r="K46" s="13" t="inlineStr">
+      <c r="K46" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-mikurunomicon</t>
         </is>
       </c>
-      <c r="L46" s="11" t="n">
+      <c r="L46" s="12" t="n">
         <v>0.001929398148148148</v>
       </c>
       <c r="M46" s="10" t="inlineStr">
@@ -2700,12 +2740,12 @@
       <c r="H47" s="9" t="inlineStr"/>
       <c r="I47" s="10" t="inlineStr"/>
       <c r="J47" s="9" t="inlineStr"/>
-      <c r="K47" s="13" t="inlineStr">
+      <c r="K47" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-singularity-1</t>
         </is>
       </c>
-      <c r="L47" s="11" t="n">
+      <c r="L47" s="12" t="n">
         <v>0.002051157407407407</v>
       </c>
       <c r="M47" s="10" t="inlineStr">
@@ -2744,12 +2784,12 @@
       <c r="H48" s="9" t="inlineStr"/>
       <c r="I48" s="10" t="inlineStr"/>
       <c r="J48" s="9" t="inlineStr"/>
-      <c r="K48" s="13" t="inlineStr">
+      <c r="K48" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-артас-сын-мой-v-20</t>
         </is>
       </c>
-      <c r="L48" s="11" t="n">
+      <c r="L48" s="12" t="n">
         <v>0.001666898148148148</v>
       </c>
       <c r="M48" s="10" t="inlineStr">
@@ -2788,12 +2828,12 @@
       <c r="H49" s="9" t="inlineStr"/>
       <c r="I49" s="10" t="inlineStr"/>
       <c r="J49" s="9" t="inlineStr"/>
-      <c r="K49" s="13" t="inlineStr">
+      <c r="K49" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-артас-сын-мой</t>
         </is>
       </c>
-      <c r="L49" s="11" t="n">
+      <c r="L49" s="12" t="n">
         <v>0.001621990740740741</v>
       </c>
       <c r="M49" s="10" t="inlineStr">
@@ -2832,12 +2872,12 @@
       <c r="H50" s="9" t="inlineStr"/>
       <c r="I50" s="10" t="inlineStr"/>
       <c r="J50" s="9" t="inlineStr"/>
-      <c r="K50" s="13" t="inlineStr">
+      <c r="K50" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-баллада-об-андратосе</t>
         </is>
       </c>
-      <c r="L50" s="11" t="n">
+      <c r="L50" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M50" s="10" t="inlineStr">
@@ -2876,12 +2916,12 @@
       <c r="H51" s="9" t="inlineStr"/>
       <c r="I51" s="10" t="inlineStr"/>
       <c r="J51" s="9" t="inlineStr"/>
-      <c r="K51" s="13" t="inlineStr">
+      <c r="K51" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-в-кругу-семьи-акт-iv</t>
         </is>
       </c>
-      <c r="L51" s="11" t="n">
+      <c r="L51" s="12" t="n">
         <v>0.002709953703703704</v>
       </c>
       <c r="M51" s="10" t="inlineStr">
@@ -2920,12 +2960,12 @@
       <c r="H52" s="9" t="inlineStr"/>
       <c r="I52" s="10" t="inlineStr"/>
       <c r="J52" s="9" t="inlineStr"/>
-      <c r="K52" s="13" t="inlineStr">
+      <c r="K52" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-владыка-черной-длани-opening</t>
         </is>
       </c>
-      <c r="L52" s="11" t="n">
+      <c r="L52" s="12" t="n">
         <v>0.002068634259259259</v>
       </c>
       <c r="M52" s="10" t="inlineStr">
@@ -2964,12 +3004,12 @@
       <c r="H53" s="9" t="inlineStr"/>
       <c r="I53" s="10" t="inlineStr"/>
       <c r="J53" s="9" t="inlineStr"/>
-      <c r="K53" s="13" t="inlineStr">
+      <c r="K53" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-воспоминание-о-лоретте</t>
         </is>
       </c>
-      <c r="L53" s="11" t="n">
+      <c r="L53" s="12" t="n">
         <v>0.002171064814814815</v>
       </c>
       <c r="M53" s="10" t="inlineStr">
@@ -3008,12 +3048,12 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="10" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr"/>
-      <c r="K54" s="13" t="inlineStr">
+      <c r="K54" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-день-кузнечного-камня</t>
         </is>
       </c>
-      <c r="L54" s="11" t="n">
+      <c r="L54" s="12" t="n">
         <v>0.001871990740740741</v>
       </c>
       <c r="M54" s="10" t="inlineStr">
@@ -3052,12 +3092,12 @@
       <c r="H55" s="9" t="inlineStr"/>
       <c r="I55" s="10" t="inlineStr"/>
       <c r="J55" s="9" t="inlineStr"/>
-      <c r="K55" s="13" t="inlineStr">
+      <c r="K55" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-дерьмадемон</t>
         </is>
       </c>
-      <c r="L55" s="11" t="n">
+      <c r="L55" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M55" s="10" t="inlineStr">
@@ -3096,12 +3136,12 @@
       <c r="H56" s="9" t="inlineStr"/>
       <c r="I56" s="10" t="inlineStr"/>
       <c r="J56" s="9" t="inlineStr"/>
-      <c r="K56" s="13" t="inlineStr">
+      <c r="K56" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-клеть-nu-metal</t>
         </is>
       </c>
-      <c r="L56" s="11" t="n">
+      <c r="L56" s="12" t="n">
         <v>0.001781134259259259</v>
       </c>
       <c r="M56" s="10" t="inlineStr">
@@ -3140,12 +3180,12 @@
       <c r="H57" s="9" t="inlineStr"/>
       <c r="I57" s="10" t="inlineStr"/>
       <c r="J57" s="9" t="inlineStr"/>
-      <c r="K57" s="13" t="inlineStr">
+      <c r="K57" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-клеть</t>
         </is>
       </c>
-      <c r="L57" s="11" t="n">
+      <c r="L57" s="12" t="n">
         <v>0.002253935185185185</v>
       </c>
       <c r="M57" s="10" t="inlineStr">
@@ -3184,12 +3224,12 @@
       <c r="H58" s="9" t="inlineStr"/>
       <c r="I58" s="10" t="inlineStr"/>
       <c r="J58" s="9" t="inlineStr"/>
-      <c r="K58" s="13" t="inlineStr">
+      <c r="K58" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-край-бесконечно-истерзанный</t>
         </is>
       </c>
-      <c r="L58" s="11" t="n">
+      <c r="L58" s="12" t="n">
         <v>0.001496412037037037</v>
       </c>
       <c r="M58" s="10" t="inlineStr">
@@ -3228,12 +3268,12 @@
       <c r="H59" s="9" t="inlineStr"/>
       <c r="I59" s="10" t="inlineStr"/>
       <c r="J59" s="9" t="inlineStr"/>
-      <c r="K59" s="13" t="inlineStr">
+      <c r="K59" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
         </is>
       </c>
-      <c r="L59" s="11" t="n">
+      <c r="L59" s="12" t="n">
         <v>0.001665046296296296</v>
       </c>
       <c r="M59" s="10" t="inlineStr">
@@ -3272,12 +3312,12 @@
       <c r="H60" s="9" t="inlineStr"/>
       <c r="I60" s="10" t="inlineStr"/>
       <c r="J60" s="9" t="inlineStr"/>
-      <c r="K60" s="13" t="inlineStr">
+      <c r="K60" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-ненависть</t>
         </is>
       </c>
-      <c r="L60" s="11" t="n">
+      <c r="L60" s="12" t="n">
         <v>0.001736689814814815</v>
       </c>
       <c r="M60" s="10" t="inlineStr">
@@ -3320,12 +3360,12 @@
       <c r="H61" s="9" t="inlineStr"/>
       <c r="I61" s="10" t="inlineStr"/>
       <c r="J61" s="9" t="inlineStr"/>
-      <c r="K61" s="13" t="inlineStr">
+      <c r="K61" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-поднимите-веки-выше</t>
         </is>
       </c>
-      <c r="L61" s="11" t="n">
+      <c r="L61" s="12" t="n">
         <v>0.002789699074074074</v>
       </c>
       <c r="M61" s="10" t="inlineStr">
@@ -3364,12 +3404,12 @@
       <c r="H62" s="9" t="inlineStr"/>
       <c r="I62" s="10" t="inlineStr"/>
       <c r="J62" s="9" t="inlineStr"/>
-      <c r="K62" s="13" t="inlineStr">
+      <c r="K62" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-полый</t>
         </is>
       </c>
-      <c r="L62" s="11" t="n">
+      <c r="L62" s="12" t="n">
         <v>0.002554398148148148</v>
       </c>
       <c r="M62" s="10" t="inlineStr">
@@ -3408,12 +3448,12 @@
       <c r="H63" s="9" t="inlineStr"/>
       <c r="I63" s="10" t="inlineStr"/>
       <c r="J63" s="9" t="inlineStr"/>
-      <c r="K63" s="13" t="inlineStr">
+      <c r="K63" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-последний-полет-бабочки</t>
         </is>
       </c>
-      <c r="L63" s="11" t="n">
+      <c r="L63" s="12" t="n">
         <v>0.001967824074074074</v>
       </c>
       <c r="M63" s="10" t="inlineStr">
@@ -3452,12 +3492,12 @@
       <c r="H64" s="9" t="inlineStr"/>
       <c r="I64" s="10" t="inlineStr"/>
       <c r="J64" s="9" t="inlineStr"/>
-      <c r="K64" s="13" t="inlineStr">
+      <c r="K64" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-проклятье-крипты-darkwave</t>
         </is>
       </c>
-      <c r="L64" s="11" t="n">
+      <c r="L64" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M64" s="10" t="inlineStr">
@@ -3496,12 +3536,12 @@
       <c r="H65" s="9" t="inlineStr"/>
       <c r="I65" s="10" t="inlineStr"/>
       <c r="J65" s="9" t="inlineStr"/>
-      <c r="K65" s="13" t="inlineStr">
+      <c r="K65" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-проклятье-крипты</t>
         </is>
       </c>
-      <c r="L65" s="11" t="n">
+      <c r="L65" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M65" s="10" t="inlineStr">
@@ -3544,12 +3584,12 @@
       <c r="H66" s="9" t="inlineStr"/>
       <c r="I66" s="10" t="inlineStr"/>
       <c r="J66" s="9" t="inlineStr"/>
-      <c r="K66" s="13" t="inlineStr">
+      <c r="K66" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-роксолана</t>
         </is>
       </c>
-      <c r="L66" s="11" t="n">
+      <c r="L66" s="12" t="n">
         <v>0.002012268518518519</v>
       </c>
       <c r="M66" s="10" t="inlineStr">
@@ -3588,12 +3628,12 @@
       <c r="H67" s="9" t="inlineStr"/>
       <c r="I67" s="10" t="inlineStr"/>
       <c r="J67" s="9" t="inlineStr"/>
-      <c r="K67" s="13" t="inlineStr">
+      <c r="K67" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-слияние-вечности</t>
         </is>
       </c>
-      <c r="L67" s="11" t="n">
+      <c r="L67" s="12" t="n">
         <v>0.001932523148148148</v>
       </c>
       <c r="M67" s="10" t="inlineStr">
@@ -3632,12 +3672,12 @@
       <c r="H68" s="9" t="inlineStr"/>
       <c r="I68" s="10" t="inlineStr"/>
       <c r="J68" s="9" t="inlineStr"/>
-      <c r="K68" s="13" t="inlineStr">
+      <c r="K68" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-терон</t>
         </is>
       </c>
-      <c r="L68" s="11" t="n">
+      <c r="L68" s="12" t="n">
         <v>0.002457523148148148</v>
       </c>
       <c r="M68" s="10" t="inlineStr">
@@ -3676,12 +3716,12 @@
       <c r="H69" s="9" t="inlineStr"/>
       <c r="I69" s="10" t="inlineStr"/>
       <c r="J69" s="9" t="inlineStr"/>
-      <c r="K69" s="13" t="inlineStr">
+      <c r="K69" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-эйдолон-1</t>
         </is>
       </c>
-      <c r="L69" s="11" t="n">
+      <c r="L69" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M69" s="10" t="inlineStr">
@@ -3720,12 +3760,12 @@
       <c r="H70" s="9" t="inlineStr"/>
       <c r="I70" s="10" t="inlineStr"/>
       <c r="J70" s="9" t="inlineStr"/>
-      <c r="K70" s="13" t="inlineStr">
+      <c r="K70" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-эйдолон-2</t>
         </is>
       </c>
-      <c r="L70" s="11" t="n">
+      <c r="L70" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M70" s="10" t="inlineStr">
@@ -3764,15 +3804,15 @@
       <c r="H71" s="9" t="inlineStr"/>
       <c r="I71" s="10" t="inlineStr"/>
       <c r="J71" s="9" t="inlineStr"/>
-      <c r="K71" s="13" t="inlineStr">
+      <c r="K71" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-эйдолон</t>
         </is>
       </c>
-      <c r="L71" s="11" t="n">
+      <c r="L71" s="12" t="n">
         <v>0.003102199074074074</v>
       </c>
-      <c r="M71" s="12" t="inlineStr">
+      <c r="M71" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -3808,12 +3848,12 @@
       <c r="H72" s="9" t="inlineStr"/>
       <c r="I72" s="10" t="inlineStr"/>
       <c r="J72" s="9" t="inlineStr"/>
-      <c r="K72" s="13" t="inlineStr">
+      <c r="K72" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-я-был-первым</t>
         </is>
       </c>
-      <c r="L72" s="11" t="n">
+      <c r="L72" s="12" t="n">
         <v>0.002488657407407407</v>
       </c>
       <c r="M72" s="10" t="inlineStr">
@@ -3852,15 +3892,15 @@
       <c r="H73" s="9" t="inlineStr"/>
       <c r="I73" s="10" t="inlineStr"/>
       <c r="J73" s="9" t="inlineStr"/>
-      <c r="K73" s="13" t="inlineStr">
+      <c r="K73" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromanta-singilarityvol2</t>
         </is>
       </c>
-      <c r="L73" s="11" t="n">
+      <c r="L73" s="12" t="n">
         <v>0.002250810185185185</v>
       </c>
-      <c r="M73" s="12" t="inlineStr">
+      <c r="M73" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -3896,12 +3936,12 @@
       <c r="H74" s="9" t="inlineStr"/>
       <c r="I74" s="10" t="inlineStr"/>
       <c r="J74" s="9" t="inlineStr"/>
-      <c r="K74" s="13" t="inlineStr">
+      <c r="K74" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/nuromanta-antipod-v-0666</t>
         </is>
       </c>
-      <c r="L74" s="11" t="n">
+      <c r="L74" s="12" t="n">
         <v>0.002544212962962963</v>
       </c>
       <c r="M74" s="10" t="inlineStr">
@@ -3936,12 +3976,12 @@
       <c r="H75" s="9" t="inlineStr"/>
       <c r="I75" s="10" t="inlineStr"/>
       <c r="J75" s="9" t="inlineStr"/>
-      <c r="K75" s="13" t="inlineStr">
+      <c r="K75" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/orchestra-de-la-poh-bain-russe</t>
         </is>
       </c>
-      <c r="L75" s="11" t="n">
+      <c r="L75" s="12" t="n">
         <v>0.001703935185185185</v>
       </c>
       <c r="M75" s="10" t="inlineStr">
@@ -3976,12 +4016,12 @@
       <c r="H76" s="9" t="inlineStr"/>
       <c r="I76" s="10" t="inlineStr"/>
       <c r="J76" s="9" t="inlineStr"/>
-      <c r="K76" s="13" t="inlineStr">
+      <c r="K76" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/powerwolf_ai_-_govnovoz_skysoundcc</t>
         </is>
       </c>
-      <c r="L76" s="11" t="n">
+      <c r="L76" s="12" t="n">
         <v>0.002279398148148148</v>
       </c>
       <c r="M76" s="10" t="inlineStr">
@@ -4016,12 +4056,12 @@
       <c r="H77" s="9" t="inlineStr"/>
       <c r="I77" s="10" t="inlineStr"/>
       <c r="J77" s="9" t="inlineStr"/>
-      <c r="K77" s="13" t="inlineStr">
+      <c r="K77" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/samhain-ball</t>
         </is>
       </c>
-      <c r="L77" s="11" t="n">
+      <c r="L77" s="12" t="n">
         <v>0.001583564814814815</v>
       </c>
       <c r="M77" s="10" t="inlineStr">
@@ -4060,15 +4100,15 @@
       <c r="H78" s="9" t="inlineStr"/>
       <c r="I78" s="10" t="inlineStr"/>
       <c r="J78" s="9" t="inlineStr"/>
-      <c r="K78" s="13" t="inlineStr">
+      <c r="K78" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/shizzard-entertaiment-skyborne</t>
         </is>
       </c>
-      <c r="L78" s="11" t="n">
+      <c r="L78" s="12" t="n">
         <v>0.002309953703703704</v>
       </c>
-      <c r="M78" s="12" t="inlineStr">
+      <c r="M78" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4108,15 +4148,15 @@
       <c r="H79" s="9" t="inlineStr"/>
       <c r="I79" s="10" t="inlineStr"/>
       <c r="J79" s="9" t="inlineStr"/>
-      <c r="K79" s="13" t="inlineStr">
+      <c r="K79" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/sleep-my-turtling</t>
         </is>
       </c>
-      <c r="L79" s="11" t="n">
+      <c r="L79" s="12" t="n">
         <v>0.004698611111111111</v>
       </c>
-      <c r="M79" s="12" t="inlineStr">
+      <c r="M79" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4156,12 +4196,12 @@
       <c r="H80" s="9" t="inlineStr"/>
       <c r="I80" s="10" t="inlineStr"/>
       <c r="J80" s="9" t="inlineStr"/>
-      <c r="K80" s="13" t="inlineStr">
+      <c r="K80" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/teron-я-был-первым-remastered</t>
         </is>
       </c>
-      <c r="L80" s="11" t="n">
+      <c r="L80" s="12" t="n">
         <v>0.002138310185185185</v>
       </c>
       <c r="M80" s="10" t="inlineStr">
@@ -4200,15 +4240,15 @@
       <c r="H81" s="9" t="inlineStr"/>
       <c r="I81" s="10" t="inlineStr"/>
       <c r="J81" s="9" t="inlineStr"/>
-      <c r="K81" s="13" t="inlineStr">
+      <c r="K81" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/traktorist-по-полям-по-полям</t>
         </is>
       </c>
-      <c r="L81" s="11" t="n">
+      <c r="L81" s="12" t="n">
         <v>0.002633333333333333</v>
       </c>
-      <c r="M81" s="12" t="inlineStr">
+      <c r="M81" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4244,12 +4284,12 @@
       <c r="H82" s="9" t="inlineStr"/>
       <c r="I82" s="10" t="inlineStr"/>
       <c r="J82" s="9" t="inlineStr"/>
-      <c r="K82" s="13" t="inlineStr">
+      <c r="K82" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/trupovoz</t>
         </is>
       </c>
-      <c r="L82" s="11" t="n">
+      <c r="L82" s="12" t="n">
         <v>0.002747222222222223</v>
       </c>
       <c r="M82" s="10" t="inlineStr">
@@ -4292,15 +4332,15 @@
       <c r="H83" s="9" t="inlineStr"/>
       <c r="I83" s="10" t="inlineStr"/>
       <c r="J83" s="9" t="inlineStr"/>
-      <c r="K83" s="13" t="inlineStr">
+      <c r="K83" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/valheim_-legacy-of-bronzebeard</t>
         </is>
       </c>
-      <c r="L83" s="11" t="n">
+      <c r="L83" s="12" t="n">
         <v>0.003588310185185185</v>
       </c>
-      <c r="M83" s="12" t="inlineStr">
+      <c r="M83" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4336,12 +4376,12 @@
       <c r="H84" s="9" t="inlineStr"/>
       <c r="I84" s="10" t="inlineStr"/>
       <c r="J84" s="9" t="inlineStr"/>
-      <c r="K84" s="13" t="inlineStr">
+      <c r="K84" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/vea-мое-болото</t>
         </is>
       </c>
-      <c r="L84" s="11" t="n">
+      <c r="L84" s="12" t="n">
         <v>0.001534953703703704</v>
       </c>
       <c r="M84" s="10" t="inlineStr">
@@ -4380,12 +4420,12 @@
       <c r="H85" s="9" t="inlineStr"/>
       <c r="I85" s="10" t="inlineStr"/>
       <c r="J85" s="9" t="inlineStr"/>
-      <c r="K85" s="13" t="inlineStr">
+      <c r="K85" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
         </is>
       </c>
-      <c r="L85" s="11" t="n">
+      <c r="L85" s="12" t="n">
         <v>0.002031134259259259</v>
       </c>
       <c r="M85" s="10" t="inlineStr">
@@ -4424,12 +4464,12 @@
       <c r="H86" s="9" t="inlineStr"/>
       <c r="I86" s="10" t="inlineStr"/>
       <c r="J86" s="9" t="inlineStr"/>
-      <c r="K86" s="13" t="inlineStr">
+      <c r="K86" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
         </is>
       </c>
-      <c r="L86" s="11" t="n">
+      <c r="L86" s="12" t="n">
         <v>0.001331712962962963</v>
       </c>
       <c r="M86" s="10" t="inlineStr">
@@ -4468,12 +4508,12 @@
       <c r="H87" s="9" t="inlineStr"/>
       <c r="I87" s="10" t="inlineStr"/>
       <c r="J87" s="9" t="inlineStr"/>
-      <c r="K87" s="13" t="inlineStr">
+      <c r="K87" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-v20</t>
         </is>
       </c>
-      <c r="L87" s="11" t="n">
+      <c r="L87" s="12" t="n">
         <v>0.001362731481481481</v>
       </c>
       <c r="M87" s="10" t="inlineStr">
@@ -4520,15 +4560,15 @@
       <c r="H88" s="9" t="inlineStr"/>
       <c r="I88" s="10" t="inlineStr"/>
       <c r="J88" s="9" t="inlineStr"/>
-      <c r="K88" s="13" t="inlineStr">
+      <c r="K88" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/wow-forever-тепло</t>
         </is>
       </c>
-      <c r="L88" s="11" t="n">
+      <c r="L88" s="12" t="n">
         <v>0.002009722222222222</v>
       </c>
-      <c r="M88" s="12" t="inlineStr">
+      <c r="M88" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4572,15 +4612,15 @@
       <c r="H89" s="9" t="inlineStr"/>
       <c r="I89" s="10" t="inlineStr"/>
       <c r="J89" s="9" t="inlineStr"/>
-      <c r="K89" s="13" t="inlineStr">
+      <c r="K89" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/wow-forever</t>
         </is>
       </c>
-      <c r="L89" s="11" t="n">
+      <c r="L89" s="12" t="n">
         <v>0.003616087962962963</v>
       </c>
-      <c r="M89" s="12" t="inlineStr">
+      <c r="M89" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4624,15 +4664,15 @@
       <c r="H90" s="9" t="inlineStr"/>
       <c r="I90" s="10" t="inlineStr"/>
       <c r="J90" s="9" t="inlineStr"/>
-      <c r="K90" s="13" t="inlineStr">
+      <c r="K90" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/а-может-просто-кисиком-стать</t>
         </is>
       </c>
-      <c r="L90" s="11" t="n">
+      <c r="L90" s="12" t="n">
         <v>0.002907175925925926</v>
       </c>
-      <c r="M90" s="12" t="inlineStr">
+      <c r="M90" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4676,15 +4716,15 @@
       <c r="H91" s="9" t="inlineStr"/>
       <c r="I91" s="10" t="inlineStr"/>
       <c r="J91" s="9" t="inlineStr"/>
-      <c r="K91" s="13" t="inlineStr">
+      <c r="K91" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/аааа-бронзби́рд…-ну-шо-это-тако́е_</t>
         </is>
       </c>
-      <c r="L91" s="11" t="n">
+      <c r="L91" s="12" t="n">
         <v>0.002066898148148148</v>
       </c>
-      <c r="M91" s="12" t="inlineStr">
+      <c r="M91" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4724,15 +4764,15 @@
       <c r="H92" s="9" t="inlineStr"/>
       <c r="I92" s="10" t="inlineStr"/>
       <c r="J92" s="9" t="inlineStr"/>
-      <c r="K92" s="13" t="inlineStr">
+      <c r="K92" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/аго́нит-в-шторме́</t>
         </is>
       </c>
-      <c r="L92" s="11" t="n">
+      <c r="L92" s="12" t="n">
         <v>0.002223611111111111</v>
       </c>
-      <c r="M92" s="12" t="inlineStr">
+      <c r="M92" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4768,15 +4808,15 @@
       <c r="H93" s="9" t="inlineStr"/>
       <c r="I93" s="10" t="inlineStr"/>
       <c r="J93" s="9" t="inlineStr"/>
-      <c r="K93" s="13" t="inlineStr">
+      <c r="K93" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/агонит-эльфийские-руины</t>
         </is>
       </c>
-      <c r="L93" s="11" t="n">
+      <c r="L93" s="12" t="n">
         <v>0.00318587962962963</v>
       </c>
-      <c r="M93" s="12" t="inlineStr">
+      <c r="M93" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4816,15 +4856,15 @@
       <c r="H94" s="9" t="inlineStr"/>
       <c r="I94" s="10" t="inlineStr"/>
       <c r="J94" s="9" t="inlineStr"/>
-      <c r="K94" s="13" t="inlineStr">
+      <c r="K94" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/айсберг-в-океане</t>
         </is>
       </c>
-      <c r="L94" s="11" t="n">
+      <c r="L94" s="12" t="n">
         <v>0.003393865740740741</v>
       </c>
-      <c r="M94" s="12" t="inlineStr">
+      <c r="M94" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4868,15 +4908,15 @@
       <c r="H95" s="9" t="inlineStr"/>
       <c r="I95" s="10" t="inlineStr"/>
       <c r="J95" s="9" t="inlineStr"/>
-      <c r="K95" s="13" t="inlineStr">
+      <c r="K95" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/алмаз-из-говнистых-глубин</t>
         </is>
       </c>
-      <c r="L95" s="11" t="n">
+      <c r="L95" s="12" t="n">
         <v>0.002481365740740741</v>
       </c>
-      <c r="M95" s="12" t="inlineStr">
+      <c r="M95" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -4916,12 +4956,12 @@
       <c r="H96" s="9" t="inlineStr"/>
       <c r="I96" s="10" t="inlineStr"/>
       <c r="J96" s="9" t="inlineStr"/>
-      <c r="K96" s="13" t="inlineStr">
+      <c r="K96" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/альтушка-для-вия-homa-brut</t>
         </is>
       </c>
-      <c r="L96" s="11" t="n">
+      <c r="L96" s="12" t="n">
         <v>0.002625</v>
       </c>
       <c r="M96" s="10" t="inlineStr">
@@ -4964,15 +5004,15 @@
       <c r="H97" s="9" t="inlineStr"/>
       <c r="I97" s="10" t="inlineStr"/>
       <c r="J97" s="9" t="inlineStr"/>
-      <c r="K97" s="13" t="inlineStr">
+      <c r="K97" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/ассуми-самочка</t>
         </is>
       </c>
-      <c r="L97" s="11" t="n">
+      <c r="L97" s="12" t="n">
         <v>0.000694675925925926</v>
       </c>
-      <c r="M97" s="12" t="inlineStr">
+      <c r="M97" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5012,15 +5052,15 @@
       <c r="H98" s="9" t="inlineStr"/>
       <c r="I98" s="10" t="inlineStr"/>
       <c r="J98" s="9" t="inlineStr"/>
-      <c r="K98" s="13" t="inlineStr">
+      <c r="K98" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/барон-ревиглаз-balenciaga</t>
         </is>
       </c>
-      <c r="L98" s="11" t="n">
+      <c r="L98" s="12" t="n">
         <v>0.003703587962962963</v>
       </c>
-      <c r="M98" s="12" t="inlineStr">
+      <c r="M98" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5060,15 +5100,15 @@
       <c r="H99" s="9" t="inlineStr"/>
       <c r="I99" s="10" t="inlineStr"/>
       <c r="J99" s="9" t="inlineStr"/>
-      <c r="K99" s="13" t="inlineStr">
+      <c r="K99" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/барон-ревиглаз-пиратский-бенгер</t>
         </is>
       </c>
-      <c r="L99" s="11" t="n">
+      <c r="L99" s="12" t="n">
         <v>0.002271064814814815</v>
       </c>
-      <c r="M99" s="12" t="inlineStr">
+      <c r="M99" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5108,15 +5148,15 @@
       <c r="H100" s="9" t="inlineStr"/>
       <c r="I100" s="10" t="inlineStr"/>
       <c r="J100" s="9" t="inlineStr"/>
-      <c r="K100" s="13" t="inlineStr">
+      <c r="K100" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/барон-ревиглаз-пиратский-косяк</t>
         </is>
       </c>
-      <c r="L100" s="11" t="n">
+      <c r="L100" s="12" t="n">
         <v>0.002089120370370371</v>
       </c>
-      <c r="M100" s="12" t="inlineStr">
+      <c r="M100" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5160,15 +5200,15 @@
       <c r="H101" s="9" t="inlineStr"/>
       <c r="I101" s="10" t="inlineStr"/>
       <c r="J101" s="9" t="inlineStr"/>
-      <c r="K101" s="13" t="inlineStr">
+      <c r="K101" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/барон-ревиглаз-feat-dj-говнокрад-закрытие-бронзбирда</t>
         </is>
       </c>
-      <c r="L101" s="11" t="n">
+      <c r="L101" s="12" t="n">
         <v>0.002136342592592593</v>
       </c>
-      <c r="M101" s="12" t="inlineStr">
+      <c r="M101" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5200,12 +5240,12 @@
       <c r="H102" s="9" t="inlineStr"/>
       <c r="I102" s="10" t="inlineStr"/>
       <c r="J102" s="9" t="inlineStr"/>
-      <c r="K102" s="13" t="inlineStr">
+      <c r="K102" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/бедство-элвиннского-леса</t>
         </is>
       </c>
-      <c r="L102" s="11" t="n">
+      <c r="L102" s="12" t="n">
         <v>0.002345601851851852</v>
       </c>
       <c r="M102" s="10" t="inlineStr">
@@ -5244,15 +5284,15 @@
       <c r="H103" s="9" t="inlineStr"/>
       <c r="I103" s="10" t="inlineStr"/>
       <c r="J103" s="9" t="inlineStr"/>
-      <c r="K103" s="13" t="inlineStr">
+      <c r="K103" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/блюз-эльфийские-руины</t>
         </is>
       </c>
-      <c r="L103" s="11" t="n">
+      <c r="L103" s="12" t="n">
         <v>0.003268055555555556</v>
       </c>
-      <c r="M103" s="12" t="inlineStr">
+      <c r="M103" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5296,15 +5336,15 @@
       <c r="H104" s="9" t="inlineStr"/>
       <c r="I104" s="10" t="inlineStr"/>
       <c r="J104" s="9" t="inlineStr"/>
-      <c r="K104" s="13" t="inlineStr">
+      <c r="K104" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/бронзбирд-закрытие</t>
         </is>
       </c>
-      <c r="L104" s="11" t="n">
+      <c r="L104" s="12" t="n">
         <v>0.002136342592592593</v>
       </c>
-      <c r="M104" s="12" t="inlineStr">
+      <c r="M104" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5344,15 +5384,15 @@
       <c r="H105" s="9" t="inlineStr"/>
       <c r="I105" s="10" t="inlineStr"/>
       <c r="J105" s="9" t="inlineStr"/>
-      <c r="K105" s="13" t="inlineStr">
+      <c r="K105" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/бухгалтер-гнилью</t>
         </is>
       </c>
-      <c r="L105" s="11" t="n">
+      <c r="L105" s="12" t="n">
         <v>0.002198842592592593</v>
       </c>
-      <c r="M105" s="12" t="inlineStr">
+      <c r="M105" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5384,12 +5424,12 @@
       <c r="H106" s="9" t="inlineStr"/>
       <c r="I106" s="10" t="inlineStr"/>
       <c r="J106" s="9" t="inlineStr"/>
-      <c r="K106" s="13" t="inlineStr">
+      <c r="K106" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/в-склеп-древний-про́клятый-темный</t>
         </is>
       </c>
-      <c r="L106" s="11" t="n">
+      <c r="L106" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M106" s="10" t="inlineStr">
@@ -5428,9 +5468,13 @@
       <c r="H107" s="9" t="inlineStr"/>
       <c r="I107" s="10" t="inlineStr"/>
       <c r="J107" s="9" t="inlineStr"/>
-      <c r="K107" s="9" t="inlineStr"/>
-      <c r="L107" s="11" t="n">
-        <v>0.002170486111111111</v>
+      <c r="K107" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/вар-прокачка</t>
+        </is>
+      </c>
+      <c r="L107" s="12" t="n">
+        <v>0.002115595868055555</v>
       </c>
       <c r="M107" s="10" t="inlineStr">
         <is>
@@ -5464,12 +5508,12 @@
       <c r="H108" s="9" t="inlineStr"/>
       <c r="I108" s="10" t="inlineStr"/>
       <c r="J108" s="9" t="inlineStr"/>
-      <c r="K108" s="13" t="inlineStr">
+      <c r="K108" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/вперед-на-брбрбрбр</t>
         </is>
       </c>
-      <c r="L108" s="11" t="n">
+      <c r="L108" s="12" t="n">
         <v>0.00276724537037037</v>
       </c>
       <c r="M108" s="10" t="inlineStr">
@@ -5504,12 +5548,12 @@
       <c r="H109" s="9" t="inlineStr"/>
       <c r="I109" s="10" t="inlineStr"/>
       <c r="J109" s="9" t="inlineStr"/>
-      <c r="K109" s="13" t="inlineStr">
+      <c r="K109" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд-v3</t>
         </is>
       </c>
-      <c r="L109" s="11" t="n">
+      <c r="L109" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M109" s="10" t="inlineStr">
@@ -5544,12 +5588,12 @@
       <c r="H110" s="9" t="inlineStr"/>
       <c r="I110" s="10" t="inlineStr"/>
       <c r="J110" s="9" t="inlineStr"/>
-      <c r="K110" s="13" t="inlineStr">
+      <c r="K110" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp</t>
         </is>
       </c>
-      <c r="L110" s="11" t="n">
+      <c r="L110" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M110" s="10" t="inlineStr">
@@ -5584,12 +5628,12 @@
       <c r="H111" s="9" t="inlineStr"/>
       <c r="I111" s="10" t="inlineStr"/>
       <c r="J111" s="9" t="inlineStr"/>
-      <c r="K111" s="13" t="inlineStr">
+      <c r="K111" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp_metal</t>
         </is>
       </c>
-      <c r="L111" s="11" t="n">
+      <c r="L111" s="12" t="n">
         <v>0.002550231481481481</v>
       </c>
       <c r="M111" s="10" t="inlineStr">
@@ -5624,12 +5668,12 @@
       <c r="H112" s="9" t="inlineStr"/>
       <c r="I112" s="10" t="inlineStr"/>
       <c r="J112" s="9" t="inlineStr"/>
-      <c r="K112" s="13" t="inlineStr">
+      <c r="K112" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд</t>
         </is>
       </c>
-      <c r="L112" s="11" t="n">
+      <c r="L112" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M112" s="10" t="inlineStr">
@@ -5672,15 +5716,15 @@
       <c r="H113" s="9" t="inlineStr"/>
       <c r="I113" s="10" t="inlineStr"/>
       <c r="J113" s="9" t="inlineStr"/>
-      <c r="K113" s="13" t="inlineStr">
+      <c r="K113" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/грехопадение</t>
         </is>
       </c>
-      <c r="L113" s="11" t="n">
+      <c r="L113" s="12" t="n">
         <v>0.003216898148148148</v>
       </c>
-      <c r="M113" s="12" t="inlineStr">
+      <c r="M113" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5720,15 +5764,15 @@
       <c r="H114" s="9" t="inlineStr"/>
       <c r="I114" s="10" t="inlineStr"/>
       <c r="J114" s="9" t="inlineStr"/>
-      <c r="K114" s="13" t="inlineStr">
+      <c r="K114" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/девять-кругов</t>
         </is>
       </c>
-      <c r="L114" s="11" t="n">
+      <c r="L114" s="12" t="n">
         <v>0.0006736111111111112</v>
       </c>
-      <c r="M114" s="12" t="inlineStr">
+      <c r="M114" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5764,15 +5808,15 @@
       <c r="H115" s="9" t="inlineStr"/>
       <c r="I115" s="10" t="inlineStr"/>
       <c r="J115" s="9" t="inlineStr"/>
-      <c r="K115" s="13" t="inlineStr">
+      <c r="K115" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/дикий-прогрев</t>
         </is>
       </c>
-      <c r="L115" s="11" t="n">
+      <c r="L115" s="12" t="n">
         <v>0.002041898148148148</v>
       </c>
-      <c r="M115" s="12" t="inlineStr">
+      <c r="M115" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5812,15 +5856,15 @@
       <c r="H116" s="9" t="inlineStr"/>
       <c r="I116" s="10" t="inlineStr"/>
       <c r="J116" s="9" t="inlineStr"/>
-      <c r="K116" s="13" t="inlineStr">
+      <c r="K116" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/димачка-вернулся-1топ</t>
         </is>
       </c>
-      <c r="L116" s="11" t="n">
+      <c r="L116" s="12" t="n">
         <v>0.002604166666666667</v>
       </c>
-      <c r="M116" s="12" t="inlineStr">
+      <c r="M116" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5852,12 +5896,12 @@
       <c r="H117" s="9" t="inlineStr"/>
       <c r="I117" s="10" t="inlineStr"/>
       <c r="J117" s="9" t="inlineStr"/>
-      <c r="K117" s="13" t="inlineStr">
+      <c r="K117" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/др-денису</t>
         </is>
       </c>
-      <c r="L117" s="11" t="n">
+      <c r="L117" s="12" t="n">
         <v>0.002172453703703704</v>
       </c>
       <c r="M117" s="10" t="inlineStr">
@@ -5896,11 +5940,15 @@
       <c r="H118" s="9" t="inlineStr"/>
       <c r="I118" s="10" t="inlineStr"/>
       <c r="J118" s="9" t="inlineStr"/>
-      <c r="K118" s="9" t="inlineStr"/>
-      <c r="L118" s="11" t="n">
+      <c r="K118" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/истории-на-гаупвахте-происшествие</t>
+        </is>
+      </c>
+      <c r="L118" s="12" t="n">
         <v>0.002083333333333333</v>
       </c>
-      <c r="M118" s="12" t="inlineStr">
+      <c r="M118" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5940,11 +5988,15 @@
       <c r="H119" s="9" t="inlineStr"/>
       <c r="I119" s="10" t="inlineStr"/>
       <c r="J119" s="9" t="inlineStr"/>
-      <c r="K119" s="9" t="inlineStr"/>
-      <c r="L119" s="11" t="n">
+      <c r="K119" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/киссик-и-рэбе-поймай-крысу</t>
+        </is>
+      </c>
+      <c r="L119" s="12" t="n">
         <v>0.002465509259259259</v>
       </c>
-      <c r="M119" s="12" t="inlineStr">
+      <c r="M119" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -5980,8 +6032,12 @@
       <c r="H120" s="9" t="inlineStr"/>
       <c r="I120" s="10" t="inlineStr"/>
       <c r="J120" s="9" t="inlineStr"/>
-      <c r="K120" s="9" t="inlineStr"/>
-      <c r="L120" s="11" t="n">
+      <c r="K120" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/копромант-коричневое-паломничество-разьеб-2</t>
+        </is>
+      </c>
+      <c r="L120" s="12" t="n">
         <v>0.002700231481481481</v>
       </c>
       <c r="M120" s="10" t="inlineStr">
@@ -6024,11 +6080,15 @@
       <c r="H121" s="9" t="inlineStr"/>
       <c r="I121" s="10" t="inlineStr"/>
       <c r="J121" s="9" t="inlineStr"/>
-      <c r="K121" s="9" t="inlineStr"/>
-      <c r="L121" s="11" t="n">
+      <c r="K121" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/копромант-коричневое-паломничество</t>
+        </is>
+      </c>
+      <c r="L121" s="12" t="n">
         <v>0.002356712962962963</v>
       </c>
-      <c r="M121" s="12" t="inlineStr">
+      <c r="M121" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6064,8 +6124,12 @@
       <c r="H122" s="9" t="inlineStr"/>
       <c r="I122" s="10" t="inlineStr"/>
       <c r="J122" s="9" t="inlineStr"/>
-      <c r="K122" s="9" t="inlineStr"/>
-      <c r="L122" s="11" t="n">
+      <c r="K122" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/копромант-миша</t>
+        </is>
+      </c>
+      <c r="L122" s="12" t="n">
         <v>0.001384953703703704</v>
       </c>
       <c r="M122" s="10" t="inlineStr">
@@ -6108,11 +6172,15 @@
       <c r="H123" s="9" t="inlineStr"/>
       <c r="I123" s="10" t="inlineStr"/>
       <c r="J123" s="9" t="inlineStr"/>
-      <c r="K123" s="9" t="inlineStr"/>
-      <c r="L123" s="11" t="n">
+      <c r="K123" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/коричневый-алмаз</t>
+        </is>
+      </c>
+      <c r="L123" s="12" t="n">
         <v>0.001556944444444445</v>
       </c>
-      <c r="M123" s="12" t="inlineStr">
+      <c r="M123" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6144,8 +6212,12 @@
       <c r="H124" s="9" t="inlineStr"/>
       <c r="I124" s="10" t="inlineStr"/>
       <c r="J124" s="9" t="inlineStr"/>
-      <c r="K124" s="9" t="inlineStr"/>
-      <c r="L124" s="11" t="n">
+      <c r="K124" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/костя-хватит-2</t>
+        </is>
+      </c>
+      <c r="L124" s="12" t="n">
         <v>0.002156712962962963</v>
       </c>
       <c r="M124" s="10" t="inlineStr">
@@ -6180,8 +6252,12 @@
       <c r="H125" s="9" t="inlineStr"/>
       <c r="I125" s="10" t="inlineStr"/>
       <c r="J125" s="9" t="inlineStr"/>
-      <c r="K125" s="9" t="inlineStr"/>
-      <c r="L125" s="11" t="n">
+      <c r="K125" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/криповая-эрилин</t>
+        </is>
+      </c>
+      <c r="L125" s="12" t="n">
         <v>0.002021296296296296</v>
       </c>
       <c r="M125" s="10" t="inlineStr">
@@ -6220,11 +6296,15 @@
       <c r="H126" s="9" t="inlineStr"/>
       <c r="I126" s="10" t="inlineStr"/>
       <c r="J126" s="9" t="inlineStr"/>
-      <c r="K126" s="9" t="inlineStr"/>
-      <c r="L126" s="11" t="n">
+      <c r="K126" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/крипота</t>
+        </is>
+      </c>
+      <c r="L126" s="12" t="n">
         <v>0.002100578703703704</v>
       </c>
-      <c r="M126" s="12" t="inlineStr">
+      <c r="M126" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6264,11 +6344,15 @@
       <c r="H127" s="9" t="inlineStr"/>
       <c r="I127" s="10" t="inlineStr"/>
       <c r="J127" s="9" t="inlineStr"/>
-      <c r="K127" s="9" t="inlineStr"/>
-      <c r="L127" s="11" t="n">
+      <c r="K127" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/кусоктора-в-мор-кадор</t>
+        </is>
+      </c>
+      <c r="L127" s="12" t="n">
         <v>0.002315277777777778</v>
       </c>
-      <c r="M127" s="12" t="inlineStr">
+      <c r="M127" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6312,11 +6396,15 @@
       <c r="H128" s="9" t="inlineStr"/>
       <c r="I128" s="10" t="inlineStr"/>
       <c r="J128" s="9" t="inlineStr"/>
-      <c r="K128" s="9" t="inlineStr"/>
-      <c r="L128" s="11" t="n">
+      <c r="K128" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/маленький-мерри</t>
+        </is>
+      </c>
+      <c r="L128" s="12" t="n">
         <v>0.002745833333333334</v>
       </c>
-      <c r="M128" s="12" t="inlineStr">
+      <c r="M128" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6356,11 +6444,15 @@
       <c r="H129" s="9" t="inlineStr"/>
       <c r="I129" s="10" t="inlineStr"/>
       <c r="J129" s="9" t="inlineStr"/>
-      <c r="K129" s="9" t="inlineStr"/>
-      <c r="L129" s="11" t="n">
+      <c r="K129" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/морнхейм-пуст-v2</t>
+        </is>
+      </c>
+      <c r="L129" s="12" t="n">
         <v>0.003111111111111111</v>
       </c>
-      <c r="M129" s="12" t="inlineStr">
+      <c r="M129" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6400,15 +6492,15 @@
       <c r="H130" s="9" t="inlineStr"/>
       <c r="I130" s="10" t="inlineStr"/>
       <c r="J130" s="9" t="inlineStr"/>
-      <c r="K130" s="13" t="inlineStr">
+      <c r="K130" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Astello/морнхейм-пуст-1</t>
         </is>
       </c>
-      <c r="L130" s="11" t="n">
+      <c r="L130" s="12" t="n">
         <v>0.003171643518518518</v>
       </c>
-      <c r="M130" s="12" t="inlineStr">
+      <c r="M130" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6440,8 +6532,12 @@
       <c r="H131" s="9" t="inlineStr"/>
       <c r="I131" s="10" t="inlineStr"/>
       <c r="J131" s="9" t="inlineStr"/>
-      <c r="K131" s="9" t="inlineStr"/>
-      <c r="L131" s="11" t="n">
+      <c r="K131" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/мы-выпьем-кровь-reverb</t>
+        </is>
+      </c>
+      <c r="L131" s="12" t="n">
         <v>0.002463541666666666</v>
       </c>
       <c r="M131" s="10" t="inlineStr">
@@ -6476,8 +6572,12 @@
       <c r="H132" s="9" t="inlineStr"/>
       <c r="I132" s="10" t="inlineStr"/>
       <c r="J132" s="9" t="inlineStr"/>
-      <c r="K132" s="9" t="inlineStr"/>
-      <c r="L132" s="11" t="n">
+      <c r="K132" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/мы-выпьем-кровь</t>
+        </is>
+      </c>
+      <c r="L132" s="12" t="n">
         <v>0.00227337962962963</v>
       </c>
       <c r="M132" s="10" t="inlineStr">
@@ -6520,11 +6620,15 @@
       <c r="H133" s="9" t="inlineStr"/>
       <c r="I133" s="10" t="inlineStr"/>
       <c r="J133" s="9" t="inlineStr"/>
-      <c r="K133" s="9" t="inlineStr"/>
-      <c r="L133" s="11" t="n">
+      <c r="K133" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/на-авиану-1</t>
+        </is>
+      </c>
+      <c r="L133" s="12" t="n">
         <v>0.00342800925925926</v>
       </c>
-      <c r="M133" s="12" t="inlineStr">
+      <c r="M133" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6564,11 +6668,15 @@
       <c r="H134" s="9" t="inlineStr"/>
       <c r="I134" s="10" t="inlineStr"/>
       <c r="J134" s="9" t="inlineStr"/>
-      <c r="K134" s="9" t="inlineStr"/>
-      <c r="L134" s="11" t="n">
+      <c r="K134" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/на-авиану-2</t>
+        </is>
+      </c>
+      <c r="L134" s="12" t="n">
         <v>0.001148611111111111</v>
       </c>
-      <c r="M134" s="12" t="inlineStr">
+      <c r="M134" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6608,11 +6716,15 @@
       <c r="H135" s="9" t="inlineStr"/>
       <c r="I135" s="10" t="inlineStr"/>
       <c r="J135" s="9" t="inlineStr"/>
-      <c r="K135" s="9" t="inlineStr"/>
-      <c r="L135" s="11" t="n">
+      <c r="K135" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/на-авиану</t>
+        </is>
+      </c>
+      <c r="L135" s="12" t="n">
         <v>0.003194675925925926</v>
       </c>
-      <c r="M135" s="12" t="inlineStr">
+      <c r="M135" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6644,8 +6756,12 @@
       <c r="H136" s="9" t="inlineStr"/>
       <c r="I136" s="10" t="inlineStr"/>
       <c r="J136" s="9" t="inlineStr"/>
-      <c r="K136" s="9" t="inlineStr"/>
-      <c r="L136" s="11" t="n">
+      <c r="K136" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/на-грани́це-у-тёмного-леса-1</t>
+        </is>
+      </c>
+      <c r="L136" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M136" s="10" t="inlineStr">
@@ -6692,11 +6808,15 @@
       <c r="H137" s="9" t="inlineStr"/>
       <c r="I137" s="10" t="inlineStr"/>
       <c r="J137" s="9" t="inlineStr"/>
-      <c r="K137" s="9" t="inlineStr"/>
-      <c r="L137" s="11" t="n">
+      <c r="K137" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/нагвар-приходи</t>
+        </is>
+      </c>
+      <c r="L137" s="12" t="n">
         <v>0.003530787037037037</v>
       </c>
-      <c r="M137" s="12" t="inlineStr">
+      <c r="M137" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6732,9 +6852,13 @@
       <c r="H138" s="9" t="inlineStr"/>
       <c r="I138" s="10" t="inlineStr"/>
       <c r="J138" s="9" t="inlineStr"/>
-      <c r="K138" s="9" t="inlineStr"/>
-      <c r="L138" s="11" t="n">
-        <v>0.002510648148148148</v>
+      <c r="K138" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/неделя-чистоты-ария-дерьмадемона</t>
+        </is>
+      </c>
+      <c r="L138" s="12" t="n">
+        <v>0.002447232719907408</v>
       </c>
       <c r="M138" s="10" t="inlineStr">
         <is>
@@ -6772,9 +6896,13 @@
       <c r="H139" s="9" t="inlineStr"/>
       <c r="I139" s="10" t="inlineStr"/>
       <c r="J139" s="9" t="inlineStr"/>
-      <c r="K139" s="9" t="inlineStr"/>
-      <c r="L139" s="11" t="n">
-        <v>0.002503587962962963</v>
+      <c r="K139" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/неделя-чистоты-клятва-рыцарей</t>
+        </is>
+      </c>
+      <c r="L139" s="12" t="n">
+        <v>0.002440245231481481</v>
       </c>
       <c r="M139" s="10" t="inlineStr">
         <is>
@@ -6812,8 +6940,12 @@
       <c r="H140" s="9" t="inlineStr"/>
       <c r="I140" s="10" t="inlineStr"/>
       <c r="J140" s="9" t="inlineStr"/>
-      <c r="K140" s="9" t="inlineStr"/>
-      <c r="L140" s="11" t="n">
+      <c r="K140" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/нейро-пох-лирика</t>
+        </is>
+      </c>
+      <c r="L140" s="12" t="n">
         <v>0.001858912037037037</v>
       </c>
       <c r="M140" s="10" t="inlineStr">
@@ -6856,11 +6988,15 @@
       <c r="H141" s="9" t="inlineStr"/>
       <c r="I141" s="10" t="inlineStr"/>
       <c r="J141" s="9" t="inlineStr"/>
-      <c r="K141" s="9" t="inlineStr"/>
-      <c r="L141" s="11" t="n">
+      <c r="K141" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/о-о-о-кача́лочка…</t>
+        </is>
+      </c>
+      <c r="L141" s="12" t="n">
         <v>0.001825810185185185</v>
       </c>
-      <c r="M141" s="12" t="inlineStr">
+      <c r="M141" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6900,11 +7036,15 @@
       <c r="H142" s="9" t="inlineStr"/>
       <c r="I142" s="10" t="inlineStr"/>
       <c r="J142" s="9" t="inlineStr"/>
-      <c r="K142" s="9" t="inlineStr"/>
-      <c r="L142" s="11" t="n">
+      <c r="K142" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/отплытие-отдать-швартовы-пляжная</t>
+        </is>
+      </c>
+      <c r="L142" s="12" t="n">
         <v>0.002286921296296296</v>
       </c>
-      <c r="M142" s="12" t="inlineStr">
+      <c r="M142" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -6936,8 +7076,12 @@
       <c r="H143" s="9" t="inlineStr"/>
       <c r="I143" s="10" t="inlineStr"/>
       <c r="J143" s="9" t="inlineStr"/>
-      <c r="K143" s="9" t="inlineStr"/>
-      <c r="L143" s="11" t="n">
+      <c r="K143" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/паладин</t>
+        </is>
+      </c>
+      <c r="L143" s="12" t="n">
         <v>0.002258912037037037</v>
       </c>
       <c r="M143" s="10" t="inlineStr">
@@ -6972,8 +7116,12 @@
       <c r="H144" s="9" t="inlineStr"/>
       <c r="I144" s="10" t="inlineStr"/>
       <c r="J144" s="9" t="inlineStr"/>
-      <c r="K144" s="9" t="inlineStr"/>
-      <c r="L144" s="11" t="n">
+      <c r="K144" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/первый-анимешный</t>
+        </is>
+      </c>
+      <c r="L144" s="12" t="n">
         <v>0.001511342592592593</v>
       </c>
       <c r="M144" s="10" t="inlineStr">
@@ -7008,8 +7156,12 @@
       <c r="H145" s="9" t="inlineStr"/>
       <c r="I145" s="10" t="inlineStr"/>
       <c r="J145" s="9" t="inlineStr"/>
-      <c r="K145" s="9" t="inlineStr"/>
-      <c r="L145" s="11" t="n">
+      <c r="K145" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/петрович-врубай-насос</t>
+        </is>
+      </c>
+      <c r="L145" s="12" t="n">
         <v>0.002451967592592592</v>
       </c>
       <c r="M145" s="10" t="inlineStr">
@@ -7044,8 +7196,12 @@
       <c r="H146" s="9" t="inlineStr"/>
       <c r="I146" s="10" t="inlineStr"/>
       <c r="J146" s="9" t="inlineStr"/>
-      <c r="K146" s="9" t="inlineStr"/>
-      <c r="L146" s="11" t="n">
+      <c r="K146" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/пир-фенхарела</t>
+        </is>
+      </c>
+      <c r="L146" s="12" t="n">
         <v>0.001581712962962963</v>
       </c>
       <c r="M146" s="10" t="inlineStr">
@@ -7080,8 +7236,12 @@
       <c r="H147" s="9" t="inlineStr"/>
       <c r="I147" s="10" t="inlineStr"/>
       <c r="J147" s="9" t="inlineStr"/>
-      <c r="K147" s="9" t="inlineStr"/>
-      <c r="L147" s="11" t="n">
+      <c r="K147" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/полные-боли</t>
+        </is>
+      </c>
+      <c r="L147" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M147" s="10" t="inlineStr">
@@ -7120,11 +7280,15 @@
       <c r="H148" s="9" t="inlineStr"/>
       <c r="I148" s="10" t="inlineStr"/>
       <c r="J148" s="9" t="inlineStr"/>
-      <c r="K148" s="9" t="inlineStr"/>
-      <c r="L148" s="11" t="n">
+      <c r="K148" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/последнее-желание</t>
+        </is>
+      </c>
+      <c r="L148" s="12" t="n">
         <v>0.004007175925925926</v>
       </c>
-      <c r="M148" s="12" t="inlineStr">
+      <c r="M148" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7164,11 +7328,15 @@
       <c r="H149" s="9" t="inlineStr"/>
       <c r="I149" s="10" t="inlineStr"/>
       <c r="J149" s="9" t="inlineStr"/>
-      <c r="K149" s="9" t="inlineStr"/>
-      <c r="L149" s="11" t="n">
+      <c r="K149" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/потные-трусики-партер</t>
+        </is>
+      </c>
+      <c r="L149" s="12" t="n">
         <v>0.002361342592592593</v>
       </c>
-      <c r="M149" s="12" t="inlineStr">
+      <c r="M149" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7208,11 +7376,15 @@
       <c r="H150" s="9" t="inlineStr"/>
       <c r="I150" s="10" t="inlineStr"/>
       <c r="J150" s="9" t="inlineStr"/>
-      <c r="K150" s="9" t="inlineStr"/>
-      <c r="L150" s="11" t="n">
+      <c r="K150" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/потные-трусики-подстрахуй-мишаню</t>
+        </is>
+      </c>
+      <c r="L150" s="12" t="n">
         <v>0.002323842592592593</v>
       </c>
-      <c r="M150" s="12" t="inlineStr">
+      <c r="M150" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7252,11 +7424,15 @@
       <c r="H151" s="9" t="inlineStr"/>
       <c r="I151" s="10" t="inlineStr"/>
       <c r="J151" s="9" t="inlineStr"/>
-      <c r="K151" s="9" t="inlineStr"/>
-      <c r="L151" s="11" t="n">
+      <c r="K151" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/потные-трусики-подтержка-важна</t>
+        </is>
+      </c>
+      <c r="L151" s="12" t="n">
         <v>0.002361342592592593</v>
       </c>
-      <c r="M151" s="12" t="inlineStr">
+      <c r="M151" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7296,11 +7472,15 @@
       <c r="H152" s="9" t="inlineStr"/>
       <c r="I152" s="10" t="inlineStr"/>
       <c r="J152" s="9" t="inlineStr"/>
-      <c r="K152" s="9" t="inlineStr"/>
-      <c r="L152" s="11" t="n">
+      <c r="K152" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/прощай-черепашка</t>
+        </is>
+      </c>
+      <c r="L152" s="12" t="n">
         <v>0.002731365740740741</v>
       </c>
-      <c r="M152" s="12" t="inlineStr">
+      <c r="M152" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7336,9 +7516,13 @@
       <c r="H153" s="9" t="inlineStr"/>
       <c r="I153" s="10" t="inlineStr"/>
       <c r="J153" s="9" t="inlineStr"/>
-      <c r="K153" s="9" t="inlineStr"/>
-      <c r="L153" s="11" t="n">
-        <v>0.002585069444444445</v>
+      <c r="K153" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/рабочий-сас-исповедь-рабаса</t>
+        </is>
+      </c>
+      <c r="L153" s="12" t="n">
+        <v>0.002519795081018519</v>
       </c>
       <c r="M153" s="10" t="inlineStr">
         <is>
@@ -7380,11 +7564,15 @@
       <c r="H154" s="9" t="inlineStr"/>
       <c r="I154" s="10" t="inlineStr"/>
       <c r="J154" s="9" t="inlineStr"/>
-      <c r="K154" s="9" t="inlineStr"/>
-      <c r="L154" s="11" t="n">
+      <c r="K154" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/роскомнадзор-бичом</t>
+        </is>
+      </c>
+      <c r="L154" s="12" t="n">
         <v>0.003325810185185186</v>
       </c>
-      <c r="M154" s="12" t="inlineStr">
+      <c r="M154" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7428,11 +7616,15 @@
       <c r="H155" s="9" t="inlineStr"/>
       <c r="I155" s="10" t="inlineStr"/>
       <c r="J155" s="9" t="inlineStr"/>
-      <c r="K155" s="9" t="inlineStr"/>
-      <c r="L155" s="11" t="n">
+      <c r="K155" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/рэп-о-сирусе-и-черном-алмазе</t>
+        </is>
+      </c>
+      <c r="L155" s="12" t="n">
         <v>0.002170833333333333</v>
       </c>
-      <c r="M155" s="12" t="inlineStr">
+      <c r="M155" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7468,11 +7660,15 @@
       <c r="H156" s="9" t="inlineStr"/>
       <c r="I156" s="10" t="inlineStr"/>
       <c r="J156" s="9" t="inlineStr"/>
-      <c r="K156" s="9" t="inlineStr"/>
-      <c r="L156" s="11" t="n">
+      <c r="K156" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/светлана-баскова-алмазик</t>
+        </is>
+      </c>
+      <c r="L156" s="12" t="n">
         <v>0.001441666666666667</v>
       </c>
-      <c r="M156" s="12" t="inlineStr">
+      <c r="M156" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7512,11 +7708,15 @@
       <c r="H157" s="9" t="inlineStr"/>
       <c r="I157" s="10" t="inlineStr"/>
       <c r="J157" s="9" t="inlineStr"/>
-      <c r="K157" s="9" t="inlineStr"/>
-      <c r="L157" s="11" t="n">
+      <c r="K157" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/светлана-баскова-комин-аут</t>
+        </is>
+      </c>
+      <c r="L157" s="12" t="n">
         <v>0.002657175925925926</v>
       </c>
-      <c r="M157" s="12" t="inlineStr">
+      <c r="M157" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7552,11 +7752,15 @@
       <c r="H158" s="9" t="inlineStr"/>
       <c r="I158" s="10" t="inlineStr"/>
       <c r="J158" s="9" t="inlineStr"/>
-      <c r="K158" s="9" t="inlineStr"/>
-      <c r="L158" s="11" t="n">
+      <c r="K158" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/свеча-горит-stigmata-сентябрь-cover-_ver-10</t>
+        </is>
+      </c>
+      <c r="L158" s="12" t="n">
         <v>0.002813310185185185</v>
       </c>
-      <c r="M158" s="12" t="inlineStr">
+      <c r="M158" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7596,11 +7800,15 @@
       <c r="H159" s="9" t="inlineStr"/>
       <c r="I159" s="10" t="inlineStr"/>
       <c r="J159" s="9" t="inlineStr"/>
-      <c r="K159" s="9" t="inlineStr"/>
-      <c r="L159" s="11" t="n">
+      <c r="K159" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/сердце-из-льдин</t>
+        </is>
+      </c>
+      <c r="L159" s="12" t="n">
         <v>0.004411921296296297</v>
       </c>
-      <c r="M159" s="12" t="inlineStr">
+      <c r="M159" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7636,8 +7844,12 @@
       <c r="H160" s="9" t="inlineStr"/>
       <c r="I160" s="10" t="inlineStr"/>
       <c r="J160" s="9" t="inlineStr"/>
-      <c r="K160" s="9" t="inlineStr"/>
-      <c r="L160" s="11" t="n">
+      <c r="K160" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/чд-капюшоны-над-головой</t>
+        </is>
+      </c>
+      <c r="L160" s="12" t="n">
         <v>0.001786689814814815</v>
       </c>
       <c r="M160" s="10" t="inlineStr">
@@ -7680,11 +7892,15 @@
       <c r="H161" s="9" t="inlineStr"/>
       <c r="I161" s="10" t="inlineStr"/>
       <c r="J161" s="9" t="inlineStr"/>
-      <c r="K161" s="9" t="inlineStr"/>
-      <c r="L161" s="11" t="n">
+      <c r="K161" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/черная-гора-1</t>
+        </is>
+      </c>
+      <c r="L161" s="12" t="n">
         <v>0.002702777777777778</v>
       </c>
-      <c r="M161" s="12" t="inlineStr">
+      <c r="M161" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7720,11 +7936,15 @@
       <c r="H162" s="9" t="inlineStr"/>
       <c r="I162" s="10" t="inlineStr"/>
       <c r="J162" s="9" t="inlineStr"/>
-      <c r="K162" s="9" t="inlineStr"/>
-      <c r="L162" s="11" t="n">
+      <c r="K162" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/черный-ворон</t>
+        </is>
+      </c>
+      <c r="L162" s="12" t="n">
         <v>0.005025810185185185</v>
       </c>
-      <c r="M162" s="12" t="inlineStr">
+      <c r="M162" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7764,11 +7984,15 @@
       <c r="H163" s="9" t="inlineStr"/>
       <c r="I163" s="10" t="inlineStr"/>
       <c r="J163" s="9" t="inlineStr"/>
-      <c r="K163" s="9" t="inlineStr"/>
-      <c r="L163" s="11" t="n">
+      <c r="K163" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/что-значит-«чёрная-длань»_</t>
+        </is>
+      </c>
+      <c r="L163" s="12" t="n">
         <v>0.003096643518518519</v>
       </c>
-      <c r="M163" s="12" t="inlineStr">
+      <c r="M163" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7804,11 +8028,15 @@
       <c r="H164" s="9" t="inlineStr"/>
       <c r="I164" s="10" t="inlineStr"/>
       <c r="J164" s="9" t="inlineStr"/>
-      <c r="K164" s="9" t="inlineStr"/>
-      <c r="L164" s="11" t="n">
+      <c r="K164" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/шалавелла-эльфийские-руины</t>
+        </is>
+      </c>
+      <c r="L164" s="12" t="n">
         <v>0.003268055555555556</v>
       </c>
-      <c r="M164" s="12" t="inlineStr">
+      <c r="M164" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7848,11 +8076,15 @@
       <c r="H165" s="9" t="inlineStr"/>
       <c r="I165" s="10" t="inlineStr"/>
       <c r="J165" s="9" t="inlineStr"/>
-      <c r="K165" s="9" t="inlineStr"/>
-      <c r="L165" s="11" t="n">
+      <c r="K165" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/шалавелла-—-маленький-парус</t>
+        </is>
+      </c>
+      <c r="L165" s="12" t="n">
         <v>0.003263310185185185</v>
       </c>
-      <c r="M165" s="12" t="inlineStr">
+      <c r="M165" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7892,11 +8124,15 @@
       <c r="H166" s="9" t="inlineStr"/>
       <c r="I166" s="10" t="inlineStr"/>
       <c r="J166" s="9" t="inlineStr"/>
-      <c r="K166" s="9" t="inlineStr"/>
-      <c r="L166" s="11" t="n">
+      <c r="K166" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/эдвархейд-погнали-на-авиану</t>
+        </is>
+      </c>
+      <c r="L166" s="12" t="n">
         <v>0.003393865740740741</v>
       </c>
-      <c r="M166" s="12" t="inlineStr">
+      <c r="M166" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7936,11 +8172,15 @@
       <c r="H167" s="9" t="inlineStr"/>
       <c r="I167" s="10" t="inlineStr"/>
       <c r="J167" s="9" t="inlineStr"/>
-      <c r="K167" s="9" t="inlineStr"/>
-      <c r="L167" s="11" t="n">
+      <c r="K167" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/эдвархейд-пора-на-авиану</t>
+        </is>
+      </c>
+      <c r="L167" s="12" t="n">
         <v>0.003414699074074074</v>
       </c>
-      <c r="M167" s="12" t="inlineStr">
+      <c r="M167" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -7980,11 +8220,15 @@
       <c r="H168" s="9" t="inlineStr"/>
       <c r="I168" s="10" t="inlineStr"/>
       <c r="J168" s="9" t="inlineStr"/>
-      <c r="K168" s="9" t="inlineStr"/>
-      <c r="L168" s="11" t="n">
+      <c r="K168" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/эра-копротеррора</t>
+        </is>
+      </c>
+      <c r="L168" s="12" t="n">
         <v>0.002011342592592593</v>
       </c>
-      <c r="M168" s="12" t="inlineStr">
+      <c r="M168" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -8020,8 +8264,12 @@
       <c r="H169" s="9" t="inlineStr"/>
       <c r="I169" s="10" t="inlineStr"/>
       <c r="J169" s="9" t="inlineStr"/>
-      <c r="K169" s="9" t="inlineStr"/>
-      <c r="L169" s="11" t="n">
+      <c r="K169" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/эрилин-я-эту-вашу-попсу-в-рот</t>
+        </is>
+      </c>
+      <c r="L169" s="12" t="n">
         <v>0.002520023148148148</v>
       </c>
       <c r="M169" s="10" t="inlineStr">
@@ -8064,11 +8312,15 @@
       <c r="H170" s="9" t="inlineStr"/>
       <c r="I170" s="10" t="inlineStr"/>
       <c r="J170" s="9" t="inlineStr"/>
-      <c r="K170" s="9" t="inlineStr"/>
-      <c r="L170" s="11" t="n">
+      <c r="K170" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/эээ…-миша́н…-миша́нчик…</t>
+        </is>
+      </c>
+      <c r="L170" s="12" t="n">
         <v>0.002081944444444444</v>
       </c>
-      <c r="M170" s="12" t="inlineStr">
+      <c r="M170" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -8108,11 +8360,15 @@
       <c r="H171" s="9" t="inlineStr"/>
       <c r="I171" s="10" t="inlineStr"/>
       <c r="J171" s="9" t="inlineStr"/>
-      <c r="K171" s="9" t="inlineStr"/>
-      <c r="L171" s="11" t="n">
+      <c r="K171" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/юлия-савичева-говновоз</t>
+        </is>
+      </c>
+      <c r="L171" s="12" t="n">
         <v>0.000984375</v>
       </c>
-      <c r="M171" s="12" t="inlineStr">
+      <c r="M171" s="13" t="inlineStr">
         <is>
           <t>Встроенная</t>
         </is>
@@ -8135,113 +8391,177 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K91" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K114" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K91" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K107" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K114" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K118" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K119" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K120" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K121" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K122" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K123" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K124" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K125" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K126" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K127" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K128" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K129" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K131" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K132" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K133" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K134" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K135" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K136" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K137" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K138" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K139" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K140" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K141" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K142" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K143" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K144" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K145" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K146" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K147" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K148" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K149" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K150" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K151" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K152" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K153" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K154" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K155" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K156" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K157" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K158" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K159" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K160" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K161" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K162" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K163" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K164" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K165" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K166" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K167" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K168" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K169" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K170" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K171" r:id="rId167"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId104"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId168"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8398,8 +8718,12 @@
       <c r="H6" s="9" t="inlineStr"/>
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="11" t="n">
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/40k-steps-to-heresy-моделист</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="n">
         <v>0.00325</v>
       </c>
       <c r="M6" s="10" t="inlineStr">
@@ -8438,8 +8762,12 @@
       <c r="H7" s="9" t="inlineStr"/>
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="9" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
-      <c r="L7" s="11" t="n">
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/_ddn-котлетка</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="n">
         <v>0.001875578703703704</v>
       </c>
       <c r="M7" s="10" t="inlineStr">
@@ -8478,8 +8806,12 @@
       <c r="H8" s="9" t="inlineStr"/>
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="11" t="n">
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/agonit-rivendare</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="n">
         <v>0.001414930555555556</v>
       </c>
       <c r="M8" s="10" t="inlineStr">
@@ -8518,8 +8850,12 @@
       <c r="H9" s="9" t="inlineStr"/>
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="9" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
-      <c r="L9" s="11" t="n">
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/baskova-зелёный-слоник-concert-version</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M9" s="10" t="inlineStr">
@@ -8554,9 +8890,13 @@
       <c r="H10" s="9" t="inlineStr"/>
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="9" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
-      <c r="L10" s="11" t="n">
-        <v>0.002170486111111111</v>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/bring-me-the-execute-прокачка</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>0.002115595868055555</v>
       </c>
       <c r="M10" s="10" t="inlineStr">
         <is>
@@ -8590,8 +8930,12 @@
       <c r="H11" s="9" t="inlineStr"/>
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="9" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
-      <c r="L11" s="11" t="n">
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/broken-shards-of-dark-talent</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="n">
         <v>0.001448842592592593</v>
       </c>
       <c r="M11" s="10" t="inlineStr">
@@ -8626,12 +8970,12 @@
       <c r="H12" s="9" t="inlineStr"/>
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="13" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/cript-cover-den-1</t>
         </is>
       </c>
-      <c r="L12" s="11" t="n">
+      <c r="L12" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M12" s="10" t="inlineStr">
@@ -8666,12 +9010,12 @@
       <c r="H13" s="9" t="inlineStr"/>
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="13" t="inlineStr">
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/cryptonit-–-проклятие-крипты</t>
         </is>
       </c>
-      <c r="L13" s="11" t="n">
+      <c r="L13" s="12" t="n">
         <v>0.002508101851851852</v>
       </c>
       <c r="M13" s="10" t="inlineStr">
@@ -8706,12 +9050,12 @@
       <c r="H14" s="9" t="inlineStr"/>
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="9" t="inlineStr"/>
-      <c r="K14" s="13" t="inlineStr">
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/digital-fury</t>
         </is>
       </c>
-      <c r="L14" s="11" t="n">
+      <c r="L14" s="12" t="n">
         <v>0.002633217592592592</v>
       </c>
       <c r="M14" s="10" t="inlineStr">
@@ -8754,12 +9098,12 @@
       <c r="H15" s="9" t="inlineStr"/>
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="13" t="inlineStr">
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
         </is>
       </c>
-      <c r="L15" s="11" t="n">
+      <c r="L15" s="12" t="n">
         <v>0.003261921296296296</v>
       </c>
       <c r="M15" s="10" t="inlineStr">
@@ -8798,12 +9142,12 @@
       <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr"/>
-      <c r="K16" s="13" t="inlineStr">
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/edovuaruhaindo-fujōnaru-te-no-kayō</t>
         </is>
       </c>
-      <c r="L16" s="11" t="n">
+      <c r="L16" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M16" s="10" t="inlineStr">
@@ -8846,12 +9190,12 @@
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="9" t="inlineStr"/>
-      <c r="K17" s="13" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/fakmod-sirus</t>
         </is>
       </c>
-      <c r="L17" s="11" t="n">
+      <c r="L17" s="12" t="n">
         <v>0.001800810185185185</v>
       </c>
       <c r="M17" s="10" t="inlineStr">
@@ -8890,12 +9234,12 @@
       <c r="H18" s="9" t="inlineStr"/>
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="9" t="inlineStr"/>
-      <c r="K18" s="13" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/fordring-о-король</t>
         </is>
       </c>
-      <c r="L18" s="11" t="n">
+      <c r="L18" s="12" t="n">
         <v>0.001606134259259259</v>
       </c>
       <c r="M18" s="10" t="inlineStr">
@@ -8938,12 +9282,12 @@
       <c r="H19" s="9" t="inlineStr"/>
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="9" t="inlineStr"/>
-      <c r="K19" s="13" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/fuckmode-wow-sirus</t>
         </is>
       </c>
-      <c r="L19" s="11" t="n">
+      <c r="L19" s="12" t="n">
         <v>0.001800578703703704</v>
       </c>
       <c r="M19" s="10" t="inlineStr">
@@ -8986,12 +9330,12 @@
       <c r="H20" s="9" t="inlineStr"/>
       <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="9" t="inlineStr"/>
-      <c r="K20" s="13" t="inlineStr">
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/greywick-hill-мэрри-хоуп</t>
         </is>
       </c>
-      <c r="L20" s="11" t="n">
+      <c r="L20" s="12" t="n">
         <v>0.00335150462962963</v>
       </c>
       <c r="M20" s="10" t="inlineStr">
@@ -9030,12 +9374,12 @@
       <c r="H21" s="9" t="inlineStr"/>
       <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="9" t="inlineStr"/>
-      <c r="K21" s="13" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/hastwood-ужас-в-вандермаре</t>
         </is>
       </c>
-      <c r="L21" s="11" t="n">
+      <c r="L21" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M21" s="10" t="inlineStr">
@@ -9070,12 +9414,12 @@
       <c r="H22" s="9" t="inlineStr"/>
       <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="9" t="inlineStr"/>
-      <c r="K22" s="13" t="inlineStr">
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/heilung_-_traust_skysoundcc</t>
         </is>
       </c>
-      <c r="L22" s="11" t="n">
+      <c r="L22" s="12" t="n">
         <v>0.006855324074074074</v>
       </c>
       <c r="M22" s="10" t="inlineStr">
@@ -9114,12 +9458,12 @@
       <c r="H23" s="9" t="inlineStr"/>
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="9" t="inlineStr"/>
-      <c r="K23" s="13" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/hestia-discordiam-sugere</t>
         </is>
       </c>
-      <c r="L23" s="11" t="n">
+      <c r="L23" s="12" t="n">
         <v>0.001683912037037037</v>
       </c>
       <c r="M23" s="10" t="inlineStr">
@@ -9162,12 +9506,12 @@
       <c r="H24" s="9" t="inlineStr"/>
       <c r="I24" s="10" t="inlineStr"/>
       <c r="J24" s="9" t="inlineStr"/>
-      <c r="K24" s="13" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/homabrut-три-ночи</t>
         </is>
       </c>
-      <c r="L24" s="11" t="n">
+      <c r="L24" s="12" t="n">
         <v>0.003156134259259259</v>
       </c>
       <c r="M24" s="10" t="inlineStr">
@@ -9206,12 +9550,12 @@
       <c r="H25" s="9" t="inlineStr"/>
       <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="9" t="inlineStr"/>
-      <c r="K25" s="13" t="inlineStr">
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/kushnerit-cursed-crypt</t>
         </is>
       </c>
-      <c r="L25" s="11" t="n">
+      <c r="L25" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M25" s="10" t="inlineStr">
@@ -9250,12 +9594,12 @@
       <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="10" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
-      <c r="K26" s="13" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/lightfair-мор-ладим</t>
         </is>
       </c>
-      <c r="L26" s="11" t="n">
+      <c r="L26" s="12" t="n">
         <v>0.002145023148148149</v>
       </c>
       <c r="M26" s="10" t="inlineStr">
@@ -9298,12 +9642,12 @@
       <c r="H27" s="9" t="inlineStr"/>
       <c r="I27" s="10" t="inlineStr"/>
       <c r="J27" s="9" t="inlineStr"/>
-      <c r="K27" s="13" t="inlineStr">
+      <c r="K27" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/morgenshtern-x-chd-саркофаг</t>
         </is>
       </c>
-      <c r="L27" s="11" t="n">
+      <c r="L27" s="12" t="n">
         <v>0.002070023148148148</v>
       </c>
       <c r="M27" s="10" t="inlineStr">
@@ -9342,12 +9686,12 @@
       <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="9" t="inlineStr"/>
-      <c r="K28" s="13" t="inlineStr">
+      <c r="K28" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/mrcrow-блю-юр</t>
         </is>
       </c>
-      <c r="L28" s="11" t="n">
+      <c r="L28" s="12" t="n">
         <v>0.002141898148148148</v>
       </c>
       <c r="M28" s="10" t="inlineStr">
@@ -9382,12 +9726,12 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="10" t="inlineStr"/>
       <c r="J29" s="9" t="inlineStr"/>
-      <c r="K29" s="13" t="inlineStr">
+      <c r="K29" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
         </is>
       </c>
-      <c r="L29" s="11" t="n">
+      <c r="L29" s="12" t="n">
         <v>0.001571064814814815</v>
       </c>
       <c r="M29" s="10" t="inlineStr">
@@ -9426,12 +9770,12 @@
       <c r="H30" s="9" t="inlineStr"/>
       <c r="I30" s="10" t="inlineStr"/>
       <c r="J30" s="9" t="inlineStr"/>
-      <c r="K30" s="13" t="inlineStr">
+      <c r="K30" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neoromant-о-король</t>
         </is>
       </c>
-      <c r="L30" s="11" t="n">
+      <c r="L30" s="12" t="n">
         <v>0.001606134259259259</v>
       </c>
       <c r="M30" s="10" t="inlineStr">
@@ -9470,12 +9814,12 @@
       <c r="H31" s="9" t="inlineStr"/>
       <c r="I31" s="10" t="inlineStr"/>
       <c r="J31" s="9" t="inlineStr"/>
-      <c r="K31" s="13" t="inlineStr">
+      <c r="K31" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-agonito-no-kokoro</t>
         </is>
       </c>
-      <c r="L31" s="11" t="n">
+      <c r="L31" s="12" t="n">
         <v>0.00226724537037037</v>
       </c>
       <c r="M31" s="10" t="inlineStr">
@@ -9514,12 +9858,12 @@
       <c r="H32" s="9" t="inlineStr"/>
       <c r="I32" s="10" t="inlineStr"/>
       <c r="J32" s="9" t="inlineStr"/>
-      <c r="K32" s="13" t="inlineStr">
+      <c r="K32" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-crypt</t>
         </is>
       </c>
-      <c r="L32" s="11" t="n">
+      <c r="L32" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M32" s="10" t="inlineStr">
@@ -9558,12 +9902,12 @@
       <c r="H33" s="9" t="inlineStr"/>
       <c r="I33" s="10" t="inlineStr"/>
       <c r="J33" s="9" t="inlineStr"/>
-      <c r="K33" s="13" t="inlineStr">
+      <c r="K33" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-destiny</t>
         </is>
       </c>
-      <c r="L33" s="11" t="n">
+      <c r="L33" s="12" t="n">
         <v>0.001761342592592593</v>
       </c>
       <c r="M33" s="10" t="inlineStr">
@@ -9606,12 +9950,12 @@
       <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="10" t="inlineStr"/>
       <c r="J34" s="9" t="inlineStr"/>
-      <c r="K34" s="13" t="inlineStr">
+      <c r="K34" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
         </is>
       </c>
-      <c r="L34" s="11" t="n">
+      <c r="L34" s="12" t="n">
         <v>0.002830324074074074</v>
       </c>
       <c r="M34" s="10" t="inlineStr">
@@ -9650,12 +9994,12 @@
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="10" t="inlineStr"/>
       <c r="J35" s="9" t="inlineStr"/>
-      <c r="K35" s="13" t="inlineStr">
+      <c r="K35" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-mikurunomicon</t>
         </is>
       </c>
-      <c r="L35" s="11" t="n">
+      <c r="L35" s="12" t="n">
         <v>0.001929398148148148</v>
       </c>
       <c r="M35" s="10" t="inlineStr">
@@ -9698,12 +10042,12 @@
       <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="10" t="inlineStr"/>
       <c r="J36" s="9" t="inlineStr"/>
-      <c r="K36" s="13" t="inlineStr">
+      <c r="K36" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-singularity-1</t>
         </is>
       </c>
-      <c r="L36" s="11" t="n">
+      <c r="L36" s="12" t="n">
         <v>0.002051157407407407</v>
       </c>
       <c r="M36" s="10" t="inlineStr">
@@ -9742,12 +10086,12 @@
       <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="10" t="inlineStr"/>
       <c r="J37" s="9" t="inlineStr"/>
-      <c r="K37" s="13" t="inlineStr">
+      <c r="K37" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-артас-сын-мой-v-20</t>
         </is>
       </c>
-      <c r="L37" s="11" t="n">
+      <c r="L37" s="12" t="n">
         <v>0.001666898148148148</v>
       </c>
       <c r="M37" s="10" t="inlineStr">
@@ -9786,12 +10130,12 @@
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="10" t="inlineStr"/>
       <c r="J38" s="9" t="inlineStr"/>
-      <c r="K38" s="13" t="inlineStr">
+      <c r="K38" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-артас-сын-мой</t>
         </is>
       </c>
-      <c r="L38" s="11" t="n">
+      <c r="L38" s="12" t="n">
         <v>0.001621990740740741</v>
       </c>
       <c r="M38" s="10" t="inlineStr">
@@ -9830,12 +10174,12 @@
       <c r="H39" s="9" t="inlineStr"/>
       <c r="I39" s="10" t="inlineStr"/>
       <c r="J39" s="9" t="inlineStr"/>
-      <c r="K39" s="13" t="inlineStr">
+      <c r="K39" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-баллада-об-андратосе</t>
         </is>
       </c>
-      <c r="L39" s="11" t="n">
+      <c r="L39" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M39" s="10" t="inlineStr">
@@ -9874,12 +10218,12 @@
       <c r="H40" s="9" t="inlineStr"/>
       <c r="I40" s="10" t="inlineStr"/>
       <c r="J40" s="9" t="inlineStr"/>
-      <c r="K40" s="13" t="inlineStr">
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-в-кругу-семьи-акт-iv</t>
         </is>
       </c>
-      <c r="L40" s="11" t="n">
+      <c r="L40" s="12" t="n">
         <v>0.002709953703703704</v>
       </c>
       <c r="M40" s="10" t="inlineStr">
@@ -9918,12 +10262,12 @@
       <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="10" t="inlineStr"/>
       <c r="J41" s="9" t="inlineStr"/>
-      <c r="K41" s="13" t="inlineStr">
+      <c r="K41" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-владыка-черной-длани-opening</t>
         </is>
       </c>
-      <c r="L41" s="11" t="n">
+      <c r="L41" s="12" t="n">
         <v>0.002068634259259259</v>
       </c>
       <c r="M41" s="10" t="inlineStr">
@@ -9962,12 +10306,12 @@
       <c r="H42" s="9" t="inlineStr"/>
       <c r="I42" s="10" t="inlineStr"/>
       <c r="J42" s="9" t="inlineStr"/>
-      <c r="K42" s="13" t="inlineStr">
+      <c r="K42" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-воспоминание-о-лоретте</t>
         </is>
       </c>
-      <c r="L42" s="11" t="n">
+      <c r="L42" s="12" t="n">
         <v>0.002171064814814815</v>
       </c>
       <c r="M42" s="10" t="inlineStr">
@@ -10006,12 +10350,12 @@
       <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="10" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr"/>
-      <c r="K43" s="13" t="inlineStr">
+      <c r="K43" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-день-кузнечного-камня</t>
         </is>
       </c>
-      <c r="L43" s="11" t="n">
+      <c r="L43" s="12" t="n">
         <v>0.001871990740740741</v>
       </c>
       <c r="M43" s="10" t="inlineStr">
@@ -10050,12 +10394,12 @@
       <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="10" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr"/>
-      <c r="K44" s="13" t="inlineStr">
+      <c r="K44" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-дерьмадемон</t>
         </is>
       </c>
-      <c r="L44" s="11" t="n">
+      <c r="L44" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M44" s="10" t="inlineStr">
@@ -10094,12 +10438,12 @@
       <c r="H45" s="9" t="inlineStr"/>
       <c r="I45" s="10" t="inlineStr"/>
       <c r="J45" s="9" t="inlineStr"/>
-      <c r="K45" s="13" t="inlineStr">
+      <c r="K45" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-клеть-nu-metal</t>
         </is>
       </c>
-      <c r="L45" s="11" t="n">
+      <c r="L45" s="12" t="n">
         <v>0.001781134259259259</v>
       </c>
       <c r="M45" s="10" t="inlineStr">
@@ -10138,12 +10482,12 @@
       <c r="H46" s="9" t="inlineStr"/>
       <c r="I46" s="10" t="inlineStr"/>
       <c r="J46" s="9" t="inlineStr"/>
-      <c r="K46" s="13" t="inlineStr">
+      <c r="K46" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-клеть</t>
         </is>
       </c>
-      <c r="L46" s="11" t="n">
+      <c r="L46" s="12" t="n">
         <v>0.002253935185185185</v>
       </c>
       <c r="M46" s="10" t="inlineStr">
@@ -10182,12 +10526,12 @@
       <c r="H47" s="9" t="inlineStr"/>
       <c r="I47" s="10" t="inlineStr"/>
       <c r="J47" s="9" t="inlineStr"/>
-      <c r="K47" s="13" t="inlineStr">
+      <c r="K47" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-край-бесконечно-истерзанный</t>
         </is>
       </c>
-      <c r="L47" s="11" t="n">
+      <c r="L47" s="12" t="n">
         <v>0.001496412037037037</v>
       </c>
       <c r="M47" s="10" t="inlineStr">
@@ -10226,12 +10570,12 @@
       <c r="H48" s="9" t="inlineStr"/>
       <c r="I48" s="10" t="inlineStr"/>
       <c r="J48" s="9" t="inlineStr"/>
-      <c r="K48" s="13" t="inlineStr">
+      <c r="K48" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
         </is>
       </c>
-      <c r="L48" s="11" t="n">
+      <c r="L48" s="12" t="n">
         <v>0.001665046296296296</v>
       </c>
       <c r="M48" s="10" t="inlineStr">
@@ -10270,12 +10614,12 @@
       <c r="H49" s="9" t="inlineStr"/>
       <c r="I49" s="10" t="inlineStr"/>
       <c r="J49" s="9" t="inlineStr"/>
-      <c r="K49" s="13" t="inlineStr">
+      <c r="K49" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-ненависть</t>
         </is>
       </c>
-      <c r="L49" s="11" t="n">
+      <c r="L49" s="12" t="n">
         <v>0.001736689814814815</v>
       </c>
       <c r="M49" s="10" t="inlineStr">
@@ -10318,12 +10662,12 @@
       <c r="H50" s="9" t="inlineStr"/>
       <c r="I50" s="10" t="inlineStr"/>
       <c r="J50" s="9" t="inlineStr"/>
-      <c r="K50" s="13" t="inlineStr">
+      <c r="K50" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-поднимите-веки-выше</t>
         </is>
       </c>
-      <c r="L50" s="11" t="n">
+      <c r="L50" s="12" t="n">
         <v>0.002789699074074074</v>
       </c>
       <c r="M50" s="10" t="inlineStr">
@@ -10362,12 +10706,12 @@
       <c r="H51" s="9" t="inlineStr"/>
       <c r="I51" s="10" t="inlineStr"/>
       <c r="J51" s="9" t="inlineStr"/>
-      <c r="K51" s="13" t="inlineStr">
+      <c r="K51" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-полый</t>
         </is>
       </c>
-      <c r="L51" s="11" t="n">
+      <c r="L51" s="12" t="n">
         <v>0.002554398148148148</v>
       </c>
       <c r="M51" s="10" t="inlineStr">
@@ -10406,12 +10750,12 @@
       <c r="H52" s="9" t="inlineStr"/>
       <c r="I52" s="10" t="inlineStr"/>
       <c r="J52" s="9" t="inlineStr"/>
-      <c r="K52" s="13" t="inlineStr">
+      <c r="K52" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-последний-полет-бабочки</t>
         </is>
       </c>
-      <c r="L52" s="11" t="n">
+      <c r="L52" s="12" t="n">
         <v>0.001967824074074074</v>
       </c>
       <c r="M52" s="10" t="inlineStr">
@@ -10450,12 +10794,12 @@
       <c r="H53" s="9" t="inlineStr"/>
       <c r="I53" s="10" t="inlineStr"/>
       <c r="J53" s="9" t="inlineStr"/>
-      <c r="K53" s="13" t="inlineStr">
+      <c r="K53" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-проклятье-крипты-darkwave</t>
         </is>
       </c>
-      <c r="L53" s="11" t="n">
+      <c r="L53" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M53" s="10" t="inlineStr">
@@ -10494,12 +10838,12 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="10" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr"/>
-      <c r="K54" s="13" t="inlineStr">
+      <c r="K54" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-проклятье-крипты</t>
         </is>
       </c>
-      <c r="L54" s="11" t="n">
+      <c r="L54" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M54" s="10" t="inlineStr">
@@ -10542,12 +10886,12 @@
       <c r="H55" s="9" t="inlineStr"/>
       <c r="I55" s="10" t="inlineStr"/>
       <c r="J55" s="9" t="inlineStr"/>
-      <c r="K55" s="13" t="inlineStr">
+      <c r="K55" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-роксолана</t>
         </is>
       </c>
-      <c r="L55" s="11" t="n">
+      <c r="L55" s="12" t="n">
         <v>0.002012268518518519</v>
       </c>
       <c r="M55" s="10" t="inlineStr">
@@ -10586,12 +10930,12 @@
       <c r="H56" s="9" t="inlineStr"/>
       <c r="I56" s="10" t="inlineStr"/>
       <c r="J56" s="9" t="inlineStr"/>
-      <c r="K56" s="13" t="inlineStr">
+      <c r="K56" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-слияние-вечности</t>
         </is>
       </c>
-      <c r="L56" s="11" t="n">
+      <c r="L56" s="12" t="n">
         <v>0.001932523148148148</v>
       </c>
       <c r="M56" s="10" t="inlineStr">
@@ -10630,12 +10974,12 @@
       <c r="H57" s="9" t="inlineStr"/>
       <c r="I57" s="10" t="inlineStr"/>
       <c r="J57" s="9" t="inlineStr"/>
-      <c r="K57" s="13" t="inlineStr">
+      <c r="K57" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-терон</t>
         </is>
       </c>
-      <c r="L57" s="11" t="n">
+      <c r="L57" s="12" t="n">
         <v>0.002457523148148148</v>
       </c>
       <c r="M57" s="10" t="inlineStr">
@@ -10674,12 +11018,12 @@
       <c r="H58" s="9" t="inlineStr"/>
       <c r="I58" s="10" t="inlineStr"/>
       <c r="J58" s="9" t="inlineStr"/>
-      <c r="K58" s="13" t="inlineStr">
+      <c r="K58" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-эйдолон-1</t>
         </is>
       </c>
-      <c r="L58" s="11" t="n">
+      <c r="L58" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M58" s="10" t="inlineStr">
@@ -10718,12 +11062,12 @@
       <c r="H59" s="9" t="inlineStr"/>
       <c r="I59" s="10" t="inlineStr"/>
       <c r="J59" s="9" t="inlineStr"/>
-      <c r="K59" s="13" t="inlineStr">
+      <c r="K59" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-эйдолон-2</t>
         </is>
       </c>
-      <c r="L59" s="11" t="n">
+      <c r="L59" s="12" t="n">
         <v>0.002783564814814815</v>
       </c>
       <c r="M59" s="10" t="inlineStr">
@@ -10762,12 +11106,12 @@
       <c r="H60" s="9" t="inlineStr"/>
       <c r="I60" s="10" t="inlineStr"/>
       <c r="J60" s="9" t="inlineStr"/>
-      <c r="K60" s="13" t="inlineStr">
+      <c r="K60" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/neuromant-я-был-первым</t>
         </is>
       </c>
-      <c r="L60" s="11" t="n">
+      <c r="L60" s="12" t="n">
         <v>0.002488657407407407</v>
       </c>
       <c r="M60" s="10" t="inlineStr">
@@ -10806,12 +11150,12 @@
       <c r="H61" s="9" t="inlineStr"/>
       <c r="I61" s="10" t="inlineStr"/>
       <c r="J61" s="9" t="inlineStr"/>
-      <c r="K61" s="13" t="inlineStr">
+      <c r="K61" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/nuromanta-antipod-v-0666</t>
         </is>
       </c>
-      <c r="L61" s="11" t="n">
+      <c r="L61" s="12" t="n">
         <v>0.002544212962962963</v>
       </c>
       <c r="M61" s="10" t="inlineStr">
@@ -10846,12 +11190,12 @@
       <c r="H62" s="9" t="inlineStr"/>
       <c r="I62" s="10" t="inlineStr"/>
       <c r="J62" s="9" t="inlineStr"/>
-      <c r="K62" s="13" t="inlineStr">
+      <c r="K62" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/orchestra-de-la-poh-bain-russe</t>
         </is>
       </c>
-      <c r="L62" s="11" t="n">
+      <c r="L62" s="12" t="n">
         <v>0.001703935185185185</v>
       </c>
       <c r="M62" s="10" t="inlineStr">
@@ -10886,12 +11230,12 @@
       <c r="H63" s="9" t="inlineStr"/>
       <c r="I63" s="10" t="inlineStr"/>
       <c r="J63" s="9" t="inlineStr"/>
-      <c r="K63" s="13" t="inlineStr">
+      <c r="K63" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/powerwolf_ai_-_govnovoz_skysoundcc</t>
         </is>
       </c>
-      <c r="L63" s="11" t="n">
+      <c r="L63" s="12" t="n">
         <v>0.002279398148148148</v>
       </c>
       <c r="M63" s="10" t="inlineStr">
@@ -10926,12 +11270,12 @@
       <c r="H64" s="9" t="inlineStr"/>
       <c r="I64" s="10" t="inlineStr"/>
       <c r="J64" s="9" t="inlineStr"/>
-      <c r="K64" s="13" t="inlineStr">
+      <c r="K64" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/samhain-ball</t>
         </is>
       </c>
-      <c r="L64" s="11" t="n">
+      <c r="L64" s="12" t="n">
         <v>0.001583564814814815</v>
       </c>
       <c r="M64" s="10" t="inlineStr">
@@ -10974,12 +11318,12 @@
       <c r="H65" s="9" t="inlineStr"/>
       <c r="I65" s="10" t="inlineStr"/>
       <c r="J65" s="9" t="inlineStr"/>
-      <c r="K65" s="13" t="inlineStr">
+      <c r="K65" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/teron-я-был-первым-remastered</t>
         </is>
       </c>
-      <c r="L65" s="11" t="n">
+      <c r="L65" s="12" t="n">
         <v>0.002138310185185185</v>
       </c>
       <c r="M65" s="10" t="inlineStr">
@@ -11018,12 +11362,12 @@
       <c r="H66" s="9" t="inlineStr"/>
       <c r="I66" s="10" t="inlineStr"/>
       <c r="J66" s="9" t="inlineStr"/>
-      <c r="K66" s="13" t="inlineStr">
+      <c r="K66" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/trupovoz</t>
         </is>
       </c>
-      <c r="L66" s="11" t="n">
+      <c r="L66" s="12" t="n">
         <v>0.002747222222222223</v>
       </c>
       <c r="M66" s="10" t="inlineStr">
@@ -11062,12 +11406,12 @@
       <c r="H67" s="9" t="inlineStr"/>
       <c r="I67" s="10" t="inlineStr"/>
       <c r="J67" s="9" t="inlineStr"/>
-      <c r="K67" s="13" t="inlineStr">
+      <c r="K67" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/vea-мое-болото</t>
         </is>
       </c>
-      <c r="L67" s="11" t="n">
+      <c r="L67" s="12" t="n">
         <v>0.001534953703703704</v>
       </c>
       <c r="M67" s="10" t="inlineStr">
@@ -11106,12 +11450,12 @@
       <c r="H68" s="9" t="inlineStr"/>
       <c r="I68" s="10" t="inlineStr"/>
       <c r="J68" s="9" t="inlineStr"/>
-      <c r="K68" s="13" t="inlineStr">
+      <c r="K68" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
         </is>
       </c>
-      <c r="L68" s="11" t="n">
+      <c r="L68" s="12" t="n">
         <v>0.002031134259259259</v>
       </c>
       <c r="M68" s="10" t="inlineStr">
@@ -11150,12 +11494,12 @@
       <c r="H69" s="9" t="inlineStr"/>
       <c r="I69" s="10" t="inlineStr"/>
       <c r="J69" s="9" t="inlineStr"/>
-      <c r="K69" s="13" t="inlineStr">
+      <c r="K69" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
         </is>
       </c>
-      <c r="L69" s="11" t="n">
+      <c r="L69" s="12" t="n">
         <v>0.001331712962962963</v>
       </c>
       <c r="M69" s="10" t="inlineStr">
@@ -11194,12 +11538,12 @@
       <c r="H70" s="9" t="inlineStr"/>
       <c r="I70" s="10" t="inlineStr"/>
       <c r="J70" s="9" t="inlineStr"/>
-      <c r="K70" s="13" t="inlineStr">
+      <c r="K70" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-v20</t>
         </is>
       </c>
-      <c r="L70" s="11" t="n">
+      <c r="L70" s="12" t="n">
         <v>0.001362731481481481</v>
       </c>
       <c r="M70" s="10" t="inlineStr">
@@ -11242,12 +11586,12 @@
       <c r="H71" s="9" t="inlineStr"/>
       <c r="I71" s="10" t="inlineStr"/>
       <c r="J71" s="9" t="inlineStr"/>
-      <c r="K71" s="13" t="inlineStr">
+      <c r="K71" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/альтушка-для-вия-homa-brut</t>
         </is>
       </c>
-      <c r="L71" s="11" t="n">
+      <c r="L71" s="12" t="n">
         <v>0.002625</v>
       </c>
       <c r="M71" s="10" t="inlineStr">
@@ -11282,12 +11626,12 @@
       <c r="H72" s="9" t="inlineStr"/>
       <c r="I72" s="10" t="inlineStr"/>
       <c r="J72" s="9" t="inlineStr"/>
-      <c r="K72" s="13" t="inlineStr">
+      <c r="K72" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/бедство-элвиннского-леса</t>
         </is>
       </c>
-      <c r="L72" s="11" t="n">
+      <c r="L72" s="12" t="n">
         <v>0.002345601851851852</v>
       </c>
       <c r="M72" s="10" t="inlineStr">
@@ -11322,12 +11666,12 @@
       <c r="H73" s="9" t="inlineStr"/>
       <c r="I73" s="10" t="inlineStr"/>
       <c r="J73" s="9" t="inlineStr"/>
-      <c r="K73" s="13" t="inlineStr">
+      <c r="K73" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/в-склеп-древний-про́клятый-темный</t>
         </is>
       </c>
-      <c r="L73" s="11" t="n">
+      <c r="L73" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M73" s="10" t="inlineStr">
@@ -11366,9 +11710,13 @@
       <c r="H74" s="9" t="inlineStr"/>
       <c r="I74" s="10" t="inlineStr"/>
       <c r="J74" s="9" t="inlineStr"/>
-      <c r="K74" s="9" t="inlineStr"/>
-      <c r="L74" s="11" t="n">
-        <v>0.002170486111111111</v>
+      <c r="K74" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/вар-прокачка</t>
+        </is>
+      </c>
+      <c r="L74" s="12" t="n">
+        <v>0.002115595868055555</v>
       </c>
       <c r="M74" s="10" t="inlineStr">
         <is>
@@ -11402,12 +11750,12 @@
       <c r="H75" s="9" t="inlineStr"/>
       <c r="I75" s="10" t="inlineStr"/>
       <c r="J75" s="9" t="inlineStr"/>
-      <c r="K75" s="13" t="inlineStr">
+      <c r="K75" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/вперед-на-брбрбрбр</t>
         </is>
       </c>
-      <c r="L75" s="11" t="n">
+      <c r="L75" s="12" t="n">
         <v>0.00276724537037037</v>
       </c>
       <c r="M75" s="10" t="inlineStr">
@@ -11442,12 +11790,12 @@
       <c r="H76" s="9" t="inlineStr"/>
       <c r="I76" s="10" t="inlineStr"/>
       <c r="J76" s="9" t="inlineStr"/>
-      <c r="K76" s="13" t="inlineStr">
+      <c r="K76" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд-v3</t>
         </is>
       </c>
-      <c r="L76" s="11" t="n">
+      <c r="L76" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M76" s="10" t="inlineStr">
@@ -11482,12 +11830,12 @@
       <c r="H77" s="9" t="inlineStr"/>
       <c r="I77" s="10" t="inlineStr"/>
       <c r="J77" s="9" t="inlineStr"/>
-      <c r="K77" s="13" t="inlineStr">
+      <c r="K77" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp</t>
         </is>
       </c>
-      <c r="L77" s="11" t="n">
+      <c r="L77" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M77" s="10" t="inlineStr">
@@ -11522,12 +11870,12 @@
       <c r="H78" s="9" t="inlineStr"/>
       <c r="I78" s="10" t="inlineStr"/>
       <c r="J78" s="9" t="inlineStr"/>
-      <c r="K78" s="13" t="inlineStr">
+      <c r="K78" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp_metal</t>
         </is>
       </c>
-      <c r="L78" s="11" t="n">
+      <c r="L78" s="12" t="n">
         <v>0.002550231481481481</v>
       </c>
       <c r="M78" s="10" t="inlineStr">
@@ -11562,12 +11910,12 @@
       <c r="H79" s="9" t="inlineStr"/>
       <c r="I79" s="10" t="inlineStr"/>
       <c r="J79" s="9" t="inlineStr"/>
-      <c r="K79" s="13" t="inlineStr">
+      <c r="K79" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/гимн-чд</t>
         </is>
       </c>
-      <c r="L79" s="11" t="n">
+      <c r="L79" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M79" s="10" t="inlineStr">
@@ -11602,12 +11950,12 @@
       <c r="H80" s="9" t="inlineStr"/>
       <c r="I80" s="10" t="inlineStr"/>
       <c r="J80" s="9" t="inlineStr"/>
-      <c r="K80" s="13" t="inlineStr">
+      <c r="K80" s="11" t="inlineStr">
         <is>
           <t>https://audius.co/Durachok/др-денису</t>
         </is>
       </c>
-      <c r="L80" s="11" t="n">
+      <c r="L80" s="12" t="n">
         <v>0.002172453703703704</v>
       </c>
       <c r="M80" s="10" t="inlineStr">
@@ -11646,8 +11994,12 @@
       <c r="H81" s="9" t="inlineStr"/>
       <c r="I81" s="10" t="inlineStr"/>
       <c r="J81" s="9" t="inlineStr"/>
-      <c r="K81" s="9" t="inlineStr"/>
-      <c r="L81" s="11" t="n">
+      <c r="K81" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/копромант-коричневое-паломничество-разьеб-2</t>
+        </is>
+      </c>
+      <c r="L81" s="12" t="n">
         <v>0.002700231481481481</v>
       </c>
       <c r="M81" s="10" t="inlineStr">
@@ -11686,8 +12038,12 @@
       <c r="H82" s="9" t="inlineStr"/>
       <c r="I82" s="10" t="inlineStr"/>
       <c r="J82" s="9" t="inlineStr"/>
-      <c r="K82" s="9" t="inlineStr"/>
-      <c r="L82" s="11" t="n">
+      <c r="K82" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/копромант-миша</t>
+        </is>
+      </c>
+      <c r="L82" s="12" t="n">
         <v>0.001384953703703704</v>
       </c>
       <c r="M82" s="10" t="inlineStr">
@@ -11722,8 +12078,12 @@
       <c r="H83" s="9" t="inlineStr"/>
       <c r="I83" s="10" t="inlineStr"/>
       <c r="J83" s="9" t="inlineStr"/>
-      <c r="K83" s="9" t="inlineStr"/>
-      <c r="L83" s="11" t="n">
+      <c r="K83" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/костя-хватит-2</t>
+        </is>
+      </c>
+      <c r="L83" s="12" t="n">
         <v>0.002156712962962963</v>
       </c>
       <c r="M83" s="10" t="inlineStr">
@@ -11758,8 +12118,12 @@
       <c r="H84" s="9" t="inlineStr"/>
       <c r="I84" s="10" t="inlineStr"/>
       <c r="J84" s="9" t="inlineStr"/>
-      <c r="K84" s="9" t="inlineStr"/>
-      <c r="L84" s="11" t="n">
+      <c r="K84" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/криповая-эрилин</t>
+        </is>
+      </c>
+      <c r="L84" s="12" t="n">
         <v>0.002021296296296296</v>
       </c>
       <c r="M84" s="10" t="inlineStr">
@@ -11794,8 +12158,12 @@
       <c r="H85" s="9" t="inlineStr"/>
       <c r="I85" s="10" t="inlineStr"/>
       <c r="J85" s="9" t="inlineStr"/>
-      <c r="K85" s="9" t="inlineStr"/>
-      <c r="L85" s="11" t="n">
+      <c r="K85" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/мы-выпьем-кровь-reverb</t>
+        </is>
+      </c>
+      <c r="L85" s="12" t="n">
         <v>0.002463541666666666</v>
       </c>
       <c r="M85" s="10" t="inlineStr">
@@ -11830,8 +12198,12 @@
       <c r="H86" s="9" t="inlineStr"/>
       <c r="I86" s="10" t="inlineStr"/>
       <c r="J86" s="9" t="inlineStr"/>
-      <c r="K86" s="9" t="inlineStr"/>
-      <c r="L86" s="11" t="n">
+      <c r="K86" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/мы-выпьем-кровь</t>
+        </is>
+      </c>
+      <c r="L86" s="12" t="n">
         <v>0.00227337962962963</v>
       </c>
       <c r="M86" s="10" t="inlineStr">
@@ -11866,8 +12238,12 @@
       <c r="H87" s="9" t="inlineStr"/>
       <c r="I87" s="10" t="inlineStr"/>
       <c r="J87" s="9" t="inlineStr"/>
-      <c r="K87" s="9" t="inlineStr"/>
-      <c r="L87" s="11" t="n">
+      <c r="K87" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/на-грани́це-у-тёмного-леса-1</t>
+        </is>
+      </c>
+      <c r="L87" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M87" s="10" t="inlineStr">
@@ -11906,9 +12282,13 @@
       <c r="H88" s="9" t="inlineStr"/>
       <c r="I88" s="10" t="inlineStr"/>
       <c r="J88" s="9" t="inlineStr"/>
-      <c r="K88" s="9" t="inlineStr"/>
-      <c r="L88" s="11" t="n">
-        <v>0.002510648148148148</v>
+      <c r="K88" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/неделя-чистоты-ария-дерьмадемона</t>
+        </is>
+      </c>
+      <c r="L88" s="12" t="n">
+        <v>0.002447232719907408</v>
       </c>
       <c r="M88" s="10" t="inlineStr">
         <is>
@@ -11946,9 +12326,13 @@
       <c r="H89" s="9" t="inlineStr"/>
       <c r="I89" s="10" t="inlineStr"/>
       <c r="J89" s="9" t="inlineStr"/>
-      <c r="K89" s="9" t="inlineStr"/>
-      <c r="L89" s="11" t="n">
-        <v>0.002503587962962963</v>
+      <c r="K89" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/неделя-чистоты-клятва-рыцарей</t>
+        </is>
+      </c>
+      <c r="L89" s="12" t="n">
+        <v>0.002440245231481481</v>
       </c>
       <c r="M89" s="10" t="inlineStr">
         <is>
@@ -11986,8 +12370,12 @@
       <c r="H90" s="9" t="inlineStr"/>
       <c r="I90" s="10" t="inlineStr"/>
       <c r="J90" s="9" t="inlineStr"/>
-      <c r="K90" s="9" t="inlineStr"/>
-      <c r="L90" s="11" t="n">
+      <c r="K90" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/нейро-пох-лирика</t>
+        </is>
+      </c>
+      <c r="L90" s="12" t="n">
         <v>0.001858912037037037</v>
       </c>
       <c r="M90" s="10" t="inlineStr">
@@ -12022,8 +12410,12 @@
       <c r="H91" s="9" t="inlineStr"/>
       <c r="I91" s="10" t="inlineStr"/>
       <c r="J91" s="9" t="inlineStr"/>
-      <c r="K91" s="9" t="inlineStr"/>
-      <c r="L91" s="11" t="n">
+      <c r="K91" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/паладин</t>
+        </is>
+      </c>
+      <c r="L91" s="12" t="n">
         <v>0.002258912037037037</v>
       </c>
       <c r="M91" s="10" t="inlineStr">
@@ -12058,8 +12450,12 @@
       <c r="H92" s="9" t="inlineStr"/>
       <c r="I92" s="10" t="inlineStr"/>
       <c r="J92" s="9" t="inlineStr"/>
-      <c r="K92" s="9" t="inlineStr"/>
-      <c r="L92" s="11" t="n">
+      <c r="K92" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/первый-анимешный</t>
+        </is>
+      </c>
+      <c r="L92" s="12" t="n">
         <v>0.001511342592592593</v>
       </c>
       <c r="M92" s="10" t="inlineStr">
@@ -12094,8 +12490,12 @@
       <c r="H93" s="9" t="inlineStr"/>
       <c r="I93" s="10" t="inlineStr"/>
       <c r="J93" s="9" t="inlineStr"/>
-      <c r="K93" s="9" t="inlineStr"/>
-      <c r="L93" s="11" t="n">
+      <c r="K93" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/петрович-врубай-насос</t>
+        </is>
+      </c>
+      <c r="L93" s="12" t="n">
         <v>0.002451967592592592</v>
       </c>
       <c r="M93" s="10" t="inlineStr">
@@ -12130,8 +12530,12 @@
       <c r="H94" s="9" t="inlineStr"/>
       <c r="I94" s="10" t="inlineStr"/>
       <c r="J94" s="9" t="inlineStr"/>
-      <c r="K94" s="9" t="inlineStr"/>
-      <c r="L94" s="11" t="n">
+      <c r="K94" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/пир-фенхарела</t>
+        </is>
+      </c>
+      <c r="L94" s="12" t="n">
         <v>0.001581712962962963</v>
       </c>
       <c r="M94" s="10" t="inlineStr">
@@ -12166,8 +12570,12 @@
       <c r="H95" s="9" t="inlineStr"/>
       <c r="I95" s="10" t="inlineStr"/>
       <c r="J95" s="9" t="inlineStr"/>
-      <c r="K95" s="9" t="inlineStr"/>
-      <c r="L95" s="11" t="n">
+      <c r="K95" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/полные-боли</t>
+        </is>
+      </c>
+      <c r="L95" s="12" t="n">
         <v>0.002778356481481481</v>
       </c>
       <c r="M95" s="10" t="inlineStr">
@@ -12206,9 +12614,13 @@
       <c r="H96" s="9" t="inlineStr"/>
       <c r="I96" s="10" t="inlineStr"/>
       <c r="J96" s="9" t="inlineStr"/>
-      <c r="K96" s="9" t="inlineStr"/>
-      <c r="L96" s="11" t="n">
-        <v>0.002585069444444445</v>
+      <c r="K96" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/рабочий-сас-исповедь-рабаса</t>
+        </is>
+      </c>
+      <c r="L96" s="12" t="n">
+        <v>0.002519795081018519</v>
       </c>
       <c r="M96" s="10" t="inlineStr">
         <is>
@@ -12246,8 +12658,12 @@
       <c r="H97" s="9" t="inlineStr"/>
       <c r="I97" s="10" t="inlineStr"/>
       <c r="J97" s="9" t="inlineStr"/>
-      <c r="K97" s="9" t="inlineStr"/>
-      <c r="L97" s="11" t="n">
+      <c r="K97" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/чд-капюшоны-над-головой</t>
+        </is>
+      </c>
+      <c r="L97" s="12" t="n">
         <v>0.001786689814814815</v>
       </c>
       <c r="M97" s="10" t="inlineStr">
@@ -12286,8 +12702,12 @@
       <c r="H98" s="9" t="inlineStr"/>
       <c r="I98" s="10" t="inlineStr"/>
       <c r="J98" s="9" t="inlineStr"/>
-      <c r="K98" s="9" t="inlineStr"/>
-      <c r="L98" s="11" t="n">
+      <c r="K98" s="11" t="inlineStr">
+        <is>
+          <t>https://audius.co/Astello/эрилин-я-эту-вашу-попсу-в-рот</t>
+        </is>
+      </c>
+      <c r="L98" s="12" t="n">
         <v>0.002520023148148148</v>
       </c>
       <c r="M98" s="10" t="inlineStr">
@@ -12309,79 +12729,104 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K91" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId95"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Point all 166 music links to Astello; migrate 102 verified Audius links
</commit_message>
<xml_diff>
--- a/Ch-D_music_catalog.xlsx
+++ b/Ch-D_music_catalog.xlsx
@@ -1334,7 +1334,7 @@
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/cript-cover-den-1</t>
+          <t>https://audius.co/Astello/cript-cover-den-1</t>
         </is>
       </c>
       <c r="L16" s="12" t="n">
@@ -1374,7 +1374,7 @@
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/cryptonit-–-проклятие-крипты</t>
+          <t>https://audius.co/Astello/cryptonit-–-проклятие-крипты</t>
         </is>
       </c>
       <c r="L17" s="12" t="n">
@@ -1414,7 +1414,7 @@
       <c r="J18" s="9" t="inlineStr"/>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/digital-fury</t>
+          <t>https://audius.co/Astello/digital-fury</t>
         </is>
       </c>
       <c r="L18" s="12" t="n">
@@ -1462,7 +1462,7 @@
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/dominus-agonetti-rivendare</t>
+          <t>https://audius.co/Astello/dominus-agonetti-rivendare</t>
         </is>
       </c>
       <c r="L19" s="12" t="n">
@@ -1510,7 +1510,7 @@
       <c r="J20" s="9" t="inlineStr"/>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
+          <t>https://audius.co/Astello/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
         </is>
       </c>
       <c r="L20" s="12" t="n">
@@ -1558,7 +1558,7 @@
       <c r="J21" s="9" t="inlineStr"/>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-ii-duetus-in-ruinis-stratholmi-aria-rivendari-et-isidis</t>
+          <t>https://audius.co/Astello/dominus-agonetti-—-opera-sessions_-part-ii-duetus-in-ruinis-stratholmi-aria-rivendari-et-isidis</t>
         </is>
       </c>
       <c r="L21" s="12" t="n">
@@ -1602,7 +1602,7 @@
       <c r="J22" s="9" t="inlineStr"/>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/edovuaruhaindo-fujōnaru-te-no-kayō</t>
+          <t>https://audius.co/Astello/edovuaruhaindo-fujōnaru-te-no-kayō</t>
         </is>
       </c>
       <c r="L22" s="12" t="n">
@@ -1650,7 +1650,7 @@
       <c r="J23" s="9" t="inlineStr"/>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/fakmod-sirus</t>
+          <t>https://audius.co/Astello/fakmod-sirus</t>
         </is>
       </c>
       <c r="L23" s="12" t="n">
@@ -1694,7 +1694,7 @@
       <c r="J24" s="9" t="inlineStr"/>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/fordring-о-король</t>
+          <t>https://audius.co/Astello/fordring-о-король</t>
         </is>
       </c>
       <c r="L24" s="12" t="n">
@@ -1742,7 +1742,7 @@
       <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/fuckmode-wow-sirus</t>
+          <t>https://audius.co/Astello/fuckmode-wow-sirus</t>
         </is>
       </c>
       <c r="L25" s="12" t="n">
@@ -1790,7 +1790,7 @@
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/greywick-hill-мэрри-хоуп</t>
+          <t>https://audius.co/Astello/greywick-hill-мэрри-хоуп</t>
         </is>
       </c>
       <c r="L26" s="12" t="n">
@@ -1834,7 +1834,7 @@
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/hastwood-владыка-черного-алмаза</t>
+          <t>https://audius.co/Astello/hastwood-владыка-черного-алмаза</t>
         </is>
       </c>
       <c r="L27" s="12" t="n">
@@ -1878,7 +1878,7 @@
       <c r="J28" s="9" t="inlineStr"/>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/hastwood-ужас-в-вандермаре</t>
+          <t>https://audius.co/Astello/hastwood-ужас-в-вандермаре</t>
         </is>
       </c>
       <c r="L28" s="12" t="n">
@@ -1918,7 +1918,7 @@
       <c r="J29" s="9" t="inlineStr"/>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/heilung_-_traust_skysoundcc</t>
+          <t>https://audius.co/Astello/heilung_-_traust_skysoundcc</t>
         </is>
       </c>
       <c r="L29" s="12" t="n">
@@ -1962,7 +1962,7 @@
       <c r="J30" s="9" t="inlineStr"/>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/hestia-discordiam-sugere</t>
+          <t>https://audius.co/Astello/hestia-discordiam-sugere</t>
         </is>
       </c>
       <c r="L30" s="12" t="n">
@@ -2010,7 +2010,7 @@
       <c r="J31" s="9" t="inlineStr"/>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/homabrut-три-ночи</t>
+          <t>https://audius.co/Astello/homabrut-три-ночи</t>
         </is>
       </c>
       <c r="L31" s="12" t="n">
@@ -2058,7 +2058,7 @@
       <c r="J32" s="9" t="inlineStr"/>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/kanye-brown-прогрелись-в-котле</t>
+          <t>https://audius.co/Astello/kanye-brown-прогрелись-в-котле</t>
         </is>
       </c>
       <c r="L32" s="12" t="n">
@@ -2102,7 +2102,7 @@
       <c r="J33" s="9" t="inlineStr"/>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/kushnerit-cursed-crypt</t>
+          <t>https://audius.co/Astello/kushnerit-cursed-crypt</t>
         </is>
       </c>
       <c r="L33" s="12" t="n">
@@ -2146,7 +2146,7 @@
       <c r="J34" s="9" t="inlineStr"/>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/lightfair-мор-ладим</t>
+          <t>https://audius.co/Astello/lightfair-мор-ладим</t>
         </is>
       </c>
       <c r="L34" s="12" t="n">
@@ -2194,7 +2194,7 @@
       <c r="J35" s="9" t="inlineStr"/>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/morgenshtern-x-chd-саркофаг</t>
+          <t>https://audius.co/Astello/morgenshtern-x-chd-саркофаг</t>
         </is>
       </c>
       <c r="L35" s="12" t="n">
@@ -2238,7 +2238,7 @@
       <c r="J36" s="9" t="inlineStr"/>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/mrcrow-блю-юр</t>
+          <t>https://audius.co/Astello/mrcrow-блю-юр</t>
         </is>
       </c>
       <c r="L36" s="12" t="n">
@@ -2294,7 +2294,7 @@
       <c r="J37" s="9" t="inlineStr"/>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/nagvar-жизнь-хороша</t>
+          <t>https://audius.co/Astello/nagvar-жизнь-хороша</t>
         </is>
       </c>
       <c r="L37" s="12" t="n">
@@ -2342,7 +2342,7 @@
       <c r="J38" s="9" t="inlineStr"/>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/nasramka-за-калич-да</t>
+          <t>https://audius.co/Astello/nasramka-за-калич-да</t>
         </is>
       </c>
       <c r="L38" s="12" t="n">
@@ -2382,7 +2382,7 @@
       <c r="J39" s="9" t="inlineStr"/>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
+          <t>https://audius.co/Astello/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
         </is>
       </c>
       <c r="L39" s="12" t="n">
@@ -2426,7 +2426,7 @@
       <c r="J40" s="9" t="inlineStr"/>
       <c r="K40" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neoromant-о-король</t>
+          <t>https://audius.co/Astello/neoromant-о-король</t>
         </is>
       </c>
       <c r="L40" s="12" t="n">
@@ -2470,7 +2470,7 @@
       <c r="J41" s="9" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-singularity</t>
+          <t>https://audius.co/Astello/neuromant-singularity</t>
         </is>
       </c>
       <c r="L41" s="12" t="n">
@@ -2514,7 +2514,7 @@
       <c r="J42" s="9" t="inlineStr"/>
       <c r="K42" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-agonito-no-kokoro</t>
+          <t>https://audius.co/Astello/neuromant-agonito-no-kokoro</t>
         </is>
       </c>
       <c r="L42" s="12" t="n">
@@ -2558,7 +2558,7 @@
       <c r="J43" s="9" t="inlineStr"/>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-crypt</t>
+          <t>https://audius.co/Astello/neuromant-crypt</t>
         </is>
       </c>
       <c r="L43" s="12" t="n">
@@ -2602,7 +2602,7 @@
       <c r="J44" s="9" t="inlineStr"/>
       <c r="K44" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-destiny</t>
+          <t>https://audius.co/Astello/neuromant-destiny</t>
         </is>
       </c>
       <c r="L44" s="12" t="n">
@@ -2650,7 +2650,7 @@
       <c r="J45" s="9" t="inlineStr"/>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
+          <t>https://audius.co/Astello/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
         </is>
       </c>
       <c r="L45" s="12" t="n">
@@ -2694,7 +2694,7 @@
       <c r="J46" s="9" t="inlineStr"/>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-mikurunomicon</t>
+          <t>https://audius.co/Astello/neuromant-mikurunomicon</t>
         </is>
       </c>
       <c r="L46" s="12" t="n">
@@ -2742,7 +2742,7 @@
       <c r="J47" s="9" t="inlineStr"/>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-singularity-1</t>
+          <t>https://audius.co/Astello/neuromant-singularity-1</t>
         </is>
       </c>
       <c r="L47" s="12" t="n">
@@ -2786,7 +2786,7 @@
       <c r="J48" s="9" t="inlineStr"/>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-артас-сын-мой-v-20</t>
+          <t>https://audius.co/Astello/neuromant-артас-сын-мой-v-20</t>
         </is>
       </c>
       <c r="L48" s="12" t="n">
@@ -2830,7 +2830,7 @@
       <c r="J49" s="9" t="inlineStr"/>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-артас-сын-мой</t>
+          <t>https://audius.co/Astello/neuromant-артас-сын-мой</t>
         </is>
       </c>
       <c r="L49" s="12" t="n">
@@ -2874,7 +2874,7 @@
       <c r="J50" s="9" t="inlineStr"/>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-баллада-об-андратосе</t>
+          <t>https://audius.co/Astello/neuromant-баллада-об-андратосе</t>
         </is>
       </c>
       <c r="L50" s="12" t="n">
@@ -2918,7 +2918,7 @@
       <c r="J51" s="9" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-в-кругу-семьи-акт-iv</t>
+          <t>https://audius.co/Astello/neuromant-в-кругу-семьи-акт-iv</t>
         </is>
       </c>
       <c r="L51" s="12" t="n">
@@ -2962,7 +2962,7 @@
       <c r="J52" s="9" t="inlineStr"/>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-владыка-черной-длани-opening</t>
+          <t>https://audius.co/Astello/neuromant-владыка-черной-длани-opening</t>
         </is>
       </c>
       <c r="L52" s="12" t="n">
@@ -3006,7 +3006,7 @@
       <c r="J53" s="9" t="inlineStr"/>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-воспоминание-о-лоретте</t>
+          <t>https://audius.co/Astello/neuromant-воспоминание-о-лоретте</t>
         </is>
       </c>
       <c r="L53" s="12" t="n">
@@ -3050,7 +3050,7 @@
       <c r="J54" s="9" t="inlineStr"/>
       <c r="K54" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-день-кузнечного-камня</t>
+          <t>https://audius.co/Astello/neuromant-день-кузнечного-камня</t>
         </is>
       </c>
       <c r="L54" s="12" t="n">
@@ -3094,7 +3094,7 @@
       <c r="J55" s="9" t="inlineStr"/>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-дерьмадемон</t>
+          <t>https://audius.co/Astello/neuromant-дерьмадемон</t>
         </is>
       </c>
       <c r="L55" s="12" t="n">
@@ -3138,7 +3138,7 @@
       <c r="J56" s="9" t="inlineStr"/>
       <c r="K56" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-клеть-nu-metal</t>
+          <t>https://audius.co/Astello/neuromant-клеть-nu-metal</t>
         </is>
       </c>
       <c r="L56" s="12" t="n">
@@ -3182,7 +3182,7 @@
       <c r="J57" s="9" t="inlineStr"/>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-клеть</t>
+          <t>https://audius.co/Astello/neuromant-клеть</t>
         </is>
       </c>
       <c r="L57" s="12" t="n">
@@ -3226,7 +3226,7 @@
       <c r="J58" s="9" t="inlineStr"/>
       <c r="K58" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-край-бесконечно-истерзанный</t>
+          <t>https://audius.co/Astello/neuromant-край-бесконечно-истерзанный</t>
         </is>
       </c>
       <c r="L58" s="12" t="n">
@@ -3270,7 +3270,7 @@
       <c r="J59" s="9" t="inlineStr"/>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
+          <t>https://audius.co/Astello/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
         </is>
       </c>
       <c r="L59" s="12" t="n">
@@ -3314,7 +3314,7 @@
       <c r="J60" s="9" t="inlineStr"/>
       <c r="K60" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-ненависть</t>
+          <t>https://audius.co/Astello/neuromant-ненависть</t>
         </is>
       </c>
       <c r="L60" s="12" t="n">
@@ -3362,7 +3362,7 @@
       <c r="J61" s="9" t="inlineStr"/>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-поднимите-веки-выше</t>
+          <t>https://audius.co/Astello/neuromant-поднимите-веки-выше</t>
         </is>
       </c>
       <c r="L61" s="12" t="n">
@@ -3406,7 +3406,7 @@
       <c r="J62" s="9" t="inlineStr"/>
       <c r="K62" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-полый</t>
+          <t>https://audius.co/Astello/neuromant-полый</t>
         </is>
       </c>
       <c r="L62" s="12" t="n">
@@ -3450,7 +3450,7 @@
       <c r="J63" s="9" t="inlineStr"/>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-последний-полет-бабочки</t>
+          <t>https://audius.co/Astello/neuromant-последний-полет-бабочки</t>
         </is>
       </c>
       <c r="L63" s="12" t="n">
@@ -3494,7 +3494,7 @@
       <c r="J64" s="9" t="inlineStr"/>
       <c r="K64" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-проклятье-крипты-darkwave</t>
+          <t>https://audius.co/Astello/neuromant-проклятье-крипты-darkwave</t>
         </is>
       </c>
       <c r="L64" s="12" t="n">
@@ -3538,7 +3538,7 @@
       <c r="J65" s="9" t="inlineStr"/>
       <c r="K65" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-проклятье-крипты</t>
+          <t>https://audius.co/Astello/neuromant-проклятье-крипты</t>
         </is>
       </c>
       <c r="L65" s="12" t="n">
@@ -3586,7 +3586,7 @@
       <c r="J66" s="9" t="inlineStr"/>
       <c r="K66" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-роксолана</t>
+          <t>https://audius.co/Astello/neuromant-роксолана</t>
         </is>
       </c>
       <c r="L66" s="12" t="n">
@@ -3630,7 +3630,7 @@
       <c r="J67" s="9" t="inlineStr"/>
       <c r="K67" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-слияние-вечности</t>
+          <t>https://audius.co/Astello/neuromant-слияние-вечности</t>
         </is>
       </c>
       <c r="L67" s="12" t="n">
@@ -3674,7 +3674,7 @@
       <c r="J68" s="9" t="inlineStr"/>
       <c r="K68" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-терон</t>
+          <t>https://audius.co/Astello/neuromant-терон</t>
         </is>
       </c>
       <c r="L68" s="12" t="n">
@@ -3718,7 +3718,7 @@
       <c r="J69" s="9" t="inlineStr"/>
       <c r="K69" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-эйдолон-1</t>
+          <t>https://audius.co/Astello/neuromant-эйдолон-1</t>
         </is>
       </c>
       <c r="L69" s="12" t="n">
@@ -3762,7 +3762,7 @@
       <c r="J70" s="9" t="inlineStr"/>
       <c r="K70" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-эйдолон-2</t>
+          <t>https://audius.co/Astello/neuromant-эйдолон-2</t>
         </is>
       </c>
       <c r="L70" s="12" t="n">
@@ -3806,7 +3806,7 @@
       <c r="J71" s="9" t="inlineStr"/>
       <c r="K71" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-эйдолон</t>
+          <t>https://audius.co/Astello/neuromant-эйдолон</t>
         </is>
       </c>
       <c r="L71" s="12" t="n">
@@ -3850,7 +3850,7 @@
       <c r="J72" s="9" t="inlineStr"/>
       <c r="K72" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-я-был-первым</t>
+          <t>https://audius.co/Astello/neuromant-я-был-первым</t>
         </is>
       </c>
       <c r="L72" s="12" t="n">
@@ -3894,7 +3894,7 @@
       <c r="J73" s="9" t="inlineStr"/>
       <c r="K73" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromanta-singilarityvol2</t>
+          <t>https://audius.co/Astello/neuromanta-singilarityvol2</t>
         </is>
       </c>
       <c r="L73" s="12" t="n">
@@ -3938,7 +3938,7 @@
       <c r="J74" s="9" t="inlineStr"/>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/nuromanta-antipod-v-0666</t>
+          <t>https://audius.co/Astello/nuromanta-antipod-v-0666</t>
         </is>
       </c>
       <c r="L74" s="12" t="n">
@@ -3978,7 +3978,7 @@
       <c r="J75" s="9" t="inlineStr"/>
       <c r="K75" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/orchestra-de-la-poh-bain-russe</t>
+          <t>https://audius.co/Astello/orchestra-de-la-poh-bain-russe</t>
         </is>
       </c>
       <c r="L75" s="12" t="n">
@@ -4018,7 +4018,7 @@
       <c r="J76" s="9" t="inlineStr"/>
       <c r="K76" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/powerwolf_ai_-_govnovoz_skysoundcc</t>
+          <t>https://audius.co/Astello/powerwolf_ai_-_govnovoz_skysoundcc</t>
         </is>
       </c>
       <c r="L76" s="12" t="n">
@@ -4058,7 +4058,7 @@
       <c r="J77" s="9" t="inlineStr"/>
       <c r="K77" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/samhain-ball</t>
+          <t>https://audius.co/Astello/samhain-ball</t>
         </is>
       </c>
       <c r="L77" s="12" t="n">
@@ -4102,7 +4102,7 @@
       <c r="J78" s="9" t="inlineStr"/>
       <c r="K78" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/shizzard-entertaiment-skyborne</t>
+          <t>https://audius.co/Astello/shizzard-entertaiment-skyborne</t>
         </is>
       </c>
       <c r="L78" s="12" t="n">
@@ -4150,7 +4150,7 @@
       <c r="J79" s="9" t="inlineStr"/>
       <c r="K79" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/sleep-my-turtling</t>
+          <t>https://audius.co/Astello/sleep-my-turtling</t>
         </is>
       </c>
       <c r="L79" s="12" t="n">
@@ -4198,7 +4198,7 @@
       <c r="J80" s="9" t="inlineStr"/>
       <c r="K80" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/teron-я-был-первым-remastered</t>
+          <t>https://audius.co/Astello/teron-я-был-первым-remastered</t>
         </is>
       </c>
       <c r="L80" s="12" t="n">
@@ -4242,7 +4242,7 @@
       <c r="J81" s="9" t="inlineStr"/>
       <c r="K81" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/traktorist-по-полям-по-полям</t>
+          <t>https://audius.co/Astello/traktorist-по-полям-по-полям</t>
         </is>
       </c>
       <c r="L81" s="12" t="n">
@@ -4286,7 +4286,7 @@
       <c r="J82" s="9" t="inlineStr"/>
       <c r="K82" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/trupovoz</t>
+          <t>https://audius.co/Astello/trupovoz</t>
         </is>
       </c>
       <c r="L82" s="12" t="n">
@@ -4334,7 +4334,7 @@
       <c r="J83" s="9" t="inlineStr"/>
       <c r="K83" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/valheim_-legacy-of-bronzebeard</t>
+          <t>https://audius.co/Astello/valheim_-legacy-of-bronzebeard</t>
         </is>
       </c>
       <c r="L83" s="12" t="n">
@@ -4378,7 +4378,7 @@
       <c r="J84" s="9" t="inlineStr"/>
       <c r="K84" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/vea-мое-болото</t>
+          <t>https://audius.co/Astello/vea-мое-болото</t>
         </is>
       </c>
       <c r="L84" s="12" t="n">
@@ -4422,7 +4422,7 @@
       <c r="J85" s="9" t="inlineStr"/>
       <c r="K85" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
+          <t>https://audius.co/Astello/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
         </is>
       </c>
       <c r="L85" s="12" t="n">
@@ -4466,7 +4466,7 @@
       <c r="J86" s="9" t="inlineStr"/>
       <c r="K86" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
+          <t>https://audius.co/Astello/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
         </is>
       </c>
       <c r="L86" s="12" t="n">
@@ -4510,7 +4510,7 @@
       <c r="J87" s="9" t="inlineStr"/>
       <c r="K87" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-v20</t>
+          <t>https://audius.co/Astello/warcrafter-вспоминаю-дни-v20</t>
         </is>
       </c>
       <c r="L87" s="12" t="n">
@@ -4562,7 +4562,7 @@
       <c r="J88" s="9" t="inlineStr"/>
       <c r="K88" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/wow-forever-тепло</t>
+          <t>https://audius.co/Astello/wow-forever-тепло</t>
         </is>
       </c>
       <c r="L88" s="12" t="n">
@@ -4614,7 +4614,7 @@
       <c r="J89" s="9" t="inlineStr"/>
       <c r="K89" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/wow-forever</t>
+          <t>https://audius.co/Astello/wow-forever</t>
         </is>
       </c>
       <c r="L89" s="12" t="n">
@@ -4666,7 +4666,7 @@
       <c r="J90" s="9" t="inlineStr"/>
       <c r="K90" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/а-может-просто-кисиком-стать</t>
+          <t>https://audius.co/Astello/а-может-просто-кисиком-стать</t>
         </is>
       </c>
       <c r="L90" s="12" t="n">
@@ -4718,7 +4718,7 @@
       <c r="J91" s="9" t="inlineStr"/>
       <c r="K91" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/аааа-бронзби́рд…-ну-шо-это-тако́е_</t>
+          <t>https://audius.co/Astello/аааа-бронзби́рд…-ну-шо-это-тако́е_</t>
         </is>
       </c>
       <c r="L91" s="12" t="n">
@@ -4766,7 +4766,7 @@
       <c r="J92" s="9" t="inlineStr"/>
       <c r="K92" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/аго́нит-в-шторме́</t>
+          <t>https://audius.co/Astello/аго́нит-в-шторме́</t>
         </is>
       </c>
       <c r="L92" s="12" t="n">
@@ -4810,7 +4810,7 @@
       <c r="J93" s="9" t="inlineStr"/>
       <c r="K93" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/агонит-эльфийские-руины</t>
+          <t>https://audius.co/Astello/агонит-эльфийские-руины</t>
         </is>
       </c>
       <c r="L93" s="12" t="n">
@@ -4858,7 +4858,7 @@
       <c r="J94" s="9" t="inlineStr"/>
       <c r="K94" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/айсберг-в-океане</t>
+          <t>https://audius.co/Astello/айсберг-в-океане</t>
         </is>
       </c>
       <c r="L94" s="12" t="n">
@@ -4910,7 +4910,7 @@
       <c r="J95" s="9" t="inlineStr"/>
       <c r="K95" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/алмаз-из-говнистых-глубин</t>
+          <t>https://audius.co/Astello/алмаз-из-говнистых-глубин</t>
         </is>
       </c>
       <c r="L95" s="12" t="n">
@@ -4958,7 +4958,7 @@
       <c r="J96" s="9" t="inlineStr"/>
       <c r="K96" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/альтушка-для-вия-homa-brut</t>
+          <t>https://audius.co/Astello/альтушка-для-вия-homa-brut</t>
         </is>
       </c>
       <c r="L96" s="12" t="n">
@@ -5006,7 +5006,7 @@
       <c r="J97" s="9" t="inlineStr"/>
       <c r="K97" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/ассуми-самочка</t>
+          <t>https://audius.co/Astello/ассуми-самочка</t>
         </is>
       </c>
       <c r="L97" s="12" t="n">
@@ -5054,7 +5054,7 @@
       <c r="J98" s="9" t="inlineStr"/>
       <c r="K98" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/барон-ревиглаз-balenciaga</t>
+          <t>https://audius.co/Astello/барон-ревиглаз-balenciaga</t>
         </is>
       </c>
       <c r="L98" s="12" t="n">
@@ -5102,7 +5102,7 @@
       <c r="J99" s="9" t="inlineStr"/>
       <c r="K99" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/барон-ревиглаз-пиратский-бенгер</t>
+          <t>https://audius.co/Astello/барон-ревиглаз-пиратский-бенгер</t>
         </is>
       </c>
       <c r="L99" s="12" t="n">
@@ -5150,7 +5150,7 @@
       <c r="J100" s="9" t="inlineStr"/>
       <c r="K100" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/барон-ревиглаз-пиратский-косяк</t>
+          <t>https://audius.co/Astello/барон-ревиглаз-пиратский-косяк</t>
         </is>
       </c>
       <c r="L100" s="12" t="n">
@@ -5202,7 +5202,7 @@
       <c r="J101" s="9" t="inlineStr"/>
       <c r="K101" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/барон-ревиглаз-feat-dj-говнокрад-закрытие-бронзбирда</t>
+          <t>https://audius.co/Astello/барон-ревиглаз-feat-dj-говнокрад-закрытие-бронзбирда</t>
         </is>
       </c>
       <c r="L101" s="12" t="n">
@@ -5242,7 +5242,7 @@
       <c r="J102" s="9" t="inlineStr"/>
       <c r="K102" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/бедство-элвиннского-леса</t>
+          <t>https://audius.co/Astello/бедство-элвиннского-леса</t>
         </is>
       </c>
       <c r="L102" s="12" t="n">
@@ -5286,7 +5286,7 @@
       <c r="J103" s="9" t="inlineStr"/>
       <c r="K103" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/блюз-эльфийские-руины</t>
+          <t>https://audius.co/Astello/блюз-эльфийские-руины</t>
         </is>
       </c>
       <c r="L103" s="12" t="n">
@@ -5338,7 +5338,7 @@
       <c r="J104" s="9" t="inlineStr"/>
       <c r="K104" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/бронзбирд-закрытие</t>
+          <t>https://audius.co/Astello/бронзбирд-закрытие</t>
         </is>
       </c>
       <c r="L104" s="12" t="n">
@@ -5386,7 +5386,7 @@
       <c r="J105" s="9" t="inlineStr"/>
       <c r="K105" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/бухгалтер-гнилью</t>
+          <t>https://audius.co/Astello/бухгалтер-гнилью</t>
         </is>
       </c>
       <c r="L105" s="12" t="n">
@@ -5426,7 +5426,7 @@
       <c r="J106" s="9" t="inlineStr"/>
       <c r="K106" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/в-склеп-древний-про́клятый-темный</t>
+          <t>https://audius.co/Astello/в-склеп-древний-про́клятый-темный</t>
         </is>
       </c>
       <c r="L106" s="12" t="n">
@@ -5470,7 +5470,7 @@
       <c r="J107" s="9" t="inlineStr"/>
       <c r="K107" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/вар-прокачка</t>
+          <t>https://audius.co/Astello/вар-прокачка</t>
         </is>
       </c>
       <c r="L107" s="12" t="n">
@@ -5510,7 +5510,7 @@
       <c r="J108" s="9" t="inlineStr"/>
       <c r="K108" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/вперед-на-брбрбрбр</t>
+          <t>https://audius.co/Astello/вперед-на-брбрбрбр</t>
         </is>
       </c>
       <c r="L108" s="12" t="n">
@@ -5550,7 +5550,7 @@
       <c r="J109" s="9" t="inlineStr"/>
       <c r="K109" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд-v3</t>
+          <t>https://audius.co/Astello/гимн-чд-v3</t>
         </is>
       </c>
       <c r="L109" s="12" t="n">
@@ -5590,7 +5590,7 @@
       <c r="J110" s="9" t="inlineStr"/>
       <c r="K110" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp</t>
+          <t>https://audius.co/Astello/гимн-чд-но-это-аниме-jp</t>
         </is>
       </c>
       <c r="L110" s="12" t="n">
@@ -5630,7 +5630,7 @@
       <c r="J111" s="9" t="inlineStr"/>
       <c r="K111" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp_metal</t>
+          <t>https://audius.co/Astello/гимн-чд-но-это-аниме-jp_metal</t>
         </is>
       </c>
       <c r="L111" s="12" t="n">
@@ -5670,7 +5670,7 @@
       <c r="J112" s="9" t="inlineStr"/>
       <c r="K112" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд</t>
+          <t>https://audius.co/Astello/гимн-чд</t>
         </is>
       </c>
       <c r="L112" s="12" t="n">
@@ -5718,7 +5718,7 @@
       <c r="J113" s="9" t="inlineStr"/>
       <c r="K113" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/грехопадение</t>
+          <t>https://audius.co/Astello/грехопадение</t>
         </is>
       </c>
       <c r="L113" s="12" t="n">
@@ -5766,7 +5766,7 @@
       <c r="J114" s="9" t="inlineStr"/>
       <c r="K114" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/девять-кругов</t>
+          <t>https://audius.co/Astello/девять-кругов</t>
         </is>
       </c>
       <c r="L114" s="12" t="n">
@@ -5810,7 +5810,7 @@
       <c r="J115" s="9" t="inlineStr"/>
       <c r="K115" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/дикий-прогрев</t>
+          <t>https://audius.co/Astello/дикий-прогрев</t>
         </is>
       </c>
       <c r="L115" s="12" t="n">
@@ -5858,7 +5858,7 @@
       <c r="J116" s="9" t="inlineStr"/>
       <c r="K116" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/димачка-вернулся-1топ</t>
+          <t>https://audius.co/Astello/димачка-вернулся-1топ</t>
         </is>
       </c>
       <c r="L116" s="12" t="n">
@@ -5898,7 +5898,7 @@
       <c r="J117" s="9" t="inlineStr"/>
       <c r="K117" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/др-денису</t>
+          <t>https://audius.co/Astello/др-денису</t>
         </is>
       </c>
       <c r="L117" s="12" t="n">
@@ -8972,7 +8972,7 @@
       <c r="J12" s="9" t="inlineStr"/>
       <c r="K12" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/cript-cover-den-1</t>
+          <t>https://audius.co/Astello/cript-cover-den-1</t>
         </is>
       </c>
       <c r="L12" s="12" t="n">
@@ -9012,7 +9012,7 @@
       <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/cryptonit-–-проклятие-крипты</t>
+          <t>https://audius.co/Astello/cryptonit-–-проклятие-крипты</t>
         </is>
       </c>
       <c r="L13" s="12" t="n">
@@ -9052,7 +9052,7 @@
       <c r="J14" s="9" t="inlineStr"/>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/digital-fury</t>
+          <t>https://audius.co/Astello/digital-fury</t>
         </is>
       </c>
       <c r="L14" s="12" t="n">
@@ -9100,7 +9100,7 @@
       <c r="J15" s="9" t="inlineStr"/>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
+          <t>https://audius.co/Astello/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
         </is>
       </c>
       <c r="L15" s="12" t="n">
@@ -9144,7 +9144,7 @@
       <c r="J16" s="9" t="inlineStr"/>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/edovuaruhaindo-fujōnaru-te-no-kayō</t>
+          <t>https://audius.co/Astello/edovuaruhaindo-fujōnaru-te-no-kayō</t>
         </is>
       </c>
       <c r="L16" s="12" t="n">
@@ -9192,7 +9192,7 @@
       <c r="J17" s="9" t="inlineStr"/>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/fakmod-sirus</t>
+          <t>https://audius.co/Astello/fakmod-sirus</t>
         </is>
       </c>
       <c r="L17" s="12" t="n">
@@ -9236,7 +9236,7 @@
       <c r="J18" s="9" t="inlineStr"/>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/fordring-о-король</t>
+          <t>https://audius.co/Astello/fordring-о-король</t>
         </is>
       </c>
       <c r="L18" s="12" t="n">
@@ -9284,7 +9284,7 @@
       <c r="J19" s="9" t="inlineStr"/>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/fuckmode-wow-sirus</t>
+          <t>https://audius.co/Astello/fuckmode-wow-sirus</t>
         </is>
       </c>
       <c r="L19" s="12" t="n">
@@ -9332,7 +9332,7 @@
       <c r="J20" s="9" t="inlineStr"/>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/greywick-hill-мэрри-хоуп</t>
+          <t>https://audius.co/Astello/greywick-hill-мэрри-хоуп</t>
         </is>
       </c>
       <c r="L20" s="12" t="n">
@@ -9376,7 +9376,7 @@
       <c r="J21" s="9" t="inlineStr"/>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/hastwood-ужас-в-вандермаре</t>
+          <t>https://audius.co/Astello/hastwood-ужас-в-вандермаре</t>
         </is>
       </c>
       <c r="L21" s="12" t="n">
@@ -9416,7 +9416,7 @@
       <c r="J22" s="9" t="inlineStr"/>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/heilung_-_traust_skysoundcc</t>
+          <t>https://audius.co/Astello/heilung_-_traust_skysoundcc</t>
         </is>
       </c>
       <c r="L22" s="12" t="n">
@@ -9460,7 +9460,7 @@
       <c r="J23" s="9" t="inlineStr"/>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/hestia-discordiam-sugere</t>
+          <t>https://audius.co/Astello/hestia-discordiam-sugere</t>
         </is>
       </c>
       <c r="L23" s="12" t="n">
@@ -9508,7 +9508,7 @@
       <c r="J24" s="9" t="inlineStr"/>
       <c r="K24" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/homabrut-три-ночи</t>
+          <t>https://audius.co/Astello/homabrut-три-ночи</t>
         </is>
       </c>
       <c r="L24" s="12" t="n">
@@ -9552,7 +9552,7 @@
       <c r="J25" s="9" t="inlineStr"/>
       <c r="K25" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/kushnerit-cursed-crypt</t>
+          <t>https://audius.co/Astello/kushnerit-cursed-crypt</t>
         </is>
       </c>
       <c r="L25" s="12" t="n">
@@ -9596,7 +9596,7 @@
       <c r="J26" s="9" t="inlineStr"/>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/lightfair-мор-ладим</t>
+          <t>https://audius.co/Astello/lightfair-мор-ладим</t>
         </is>
       </c>
       <c r="L26" s="12" t="n">
@@ -9644,7 +9644,7 @@
       <c r="J27" s="9" t="inlineStr"/>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/morgenshtern-x-chd-саркофаг</t>
+          <t>https://audius.co/Astello/morgenshtern-x-chd-саркофаг</t>
         </is>
       </c>
       <c r="L27" s="12" t="n">
@@ -9688,7 +9688,7 @@
       <c r="J28" s="9" t="inlineStr"/>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/mrcrow-блю-юр</t>
+          <t>https://audius.co/Astello/mrcrow-блю-юр</t>
         </is>
       </c>
       <c r="L28" s="12" t="n">
@@ -9728,7 +9728,7 @@
       <c r="J29" s="9" t="inlineStr"/>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
+          <t>https://audius.co/Astello/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
         </is>
       </c>
       <c r="L29" s="12" t="n">
@@ -9772,7 +9772,7 @@
       <c r="J30" s="9" t="inlineStr"/>
       <c r="K30" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neoromant-о-король</t>
+          <t>https://audius.co/Astello/neoromant-о-король</t>
         </is>
       </c>
       <c r="L30" s="12" t="n">
@@ -9816,7 +9816,7 @@
       <c r="J31" s="9" t="inlineStr"/>
       <c r="K31" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-agonito-no-kokoro</t>
+          <t>https://audius.co/Astello/neuromant-agonito-no-kokoro</t>
         </is>
       </c>
       <c r="L31" s="12" t="n">
@@ -9860,7 +9860,7 @@
       <c r="J32" s="9" t="inlineStr"/>
       <c r="K32" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-crypt</t>
+          <t>https://audius.co/Astello/neuromant-crypt</t>
         </is>
       </c>
       <c r="L32" s="12" t="n">
@@ -9904,7 +9904,7 @@
       <c r="J33" s="9" t="inlineStr"/>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-destiny</t>
+          <t>https://audius.co/Astello/neuromant-destiny</t>
         </is>
       </c>
       <c r="L33" s="12" t="n">
@@ -9952,7 +9952,7 @@
       <c r="J34" s="9" t="inlineStr"/>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
+          <t>https://audius.co/Astello/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
         </is>
       </c>
       <c r="L34" s="12" t="n">
@@ -9996,7 +9996,7 @@
       <c r="J35" s="9" t="inlineStr"/>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-mikurunomicon</t>
+          <t>https://audius.co/Astello/neuromant-mikurunomicon</t>
         </is>
       </c>
       <c r="L35" s="12" t="n">
@@ -10044,7 +10044,7 @@
       <c r="J36" s="9" t="inlineStr"/>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-singularity-1</t>
+          <t>https://audius.co/Astello/neuromant-singularity-1</t>
         </is>
       </c>
       <c r="L36" s="12" t="n">
@@ -10088,7 +10088,7 @@
       <c r="J37" s="9" t="inlineStr"/>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-артас-сын-мой-v-20</t>
+          <t>https://audius.co/Astello/neuromant-артас-сын-мой-v-20</t>
         </is>
       </c>
       <c r="L37" s="12" t="n">
@@ -10132,7 +10132,7 @@
       <c r="J38" s="9" t="inlineStr"/>
       <c r="K38" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-артас-сын-мой</t>
+          <t>https://audius.co/Astello/neuromant-артас-сын-мой</t>
         </is>
       </c>
       <c r="L38" s="12" t="n">
@@ -10176,7 +10176,7 @@
       <c r="J39" s="9" t="inlineStr"/>
       <c r="K39" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-баллада-об-андратосе</t>
+          <t>https://audius.co/Astello/neuromant-баллада-об-андратосе</t>
         </is>
       </c>
       <c r="L39" s="12" t="n">
@@ -10220,7 +10220,7 @@
       <c r="J40" s="9" t="inlineStr"/>
       <c r="K40" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-в-кругу-семьи-акт-iv</t>
+          <t>https://audius.co/Astello/neuromant-в-кругу-семьи-акт-iv</t>
         </is>
       </c>
       <c r="L40" s="12" t="n">
@@ -10264,7 +10264,7 @@
       <c r="J41" s="9" t="inlineStr"/>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-владыка-черной-длани-opening</t>
+          <t>https://audius.co/Astello/neuromant-владыка-черной-длани-opening</t>
         </is>
       </c>
       <c r="L41" s="12" t="n">
@@ -10308,7 +10308,7 @@
       <c r="J42" s="9" t="inlineStr"/>
       <c r="K42" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-воспоминание-о-лоретте</t>
+          <t>https://audius.co/Astello/neuromant-воспоминание-о-лоретте</t>
         </is>
       </c>
       <c r="L42" s="12" t="n">
@@ -10352,7 +10352,7 @@
       <c r="J43" s="9" t="inlineStr"/>
       <c r="K43" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-день-кузнечного-камня</t>
+          <t>https://audius.co/Astello/neuromant-день-кузнечного-камня</t>
         </is>
       </c>
       <c r="L43" s="12" t="n">
@@ -10396,7 +10396,7 @@
       <c r="J44" s="9" t="inlineStr"/>
       <c r="K44" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-дерьмадемон</t>
+          <t>https://audius.co/Astello/neuromant-дерьмадемон</t>
         </is>
       </c>
       <c r="L44" s="12" t="n">
@@ -10440,7 +10440,7 @@
       <c r="J45" s="9" t="inlineStr"/>
       <c r="K45" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-клеть-nu-metal</t>
+          <t>https://audius.co/Astello/neuromant-клеть-nu-metal</t>
         </is>
       </c>
       <c r="L45" s="12" t="n">
@@ -10484,7 +10484,7 @@
       <c r="J46" s="9" t="inlineStr"/>
       <c r="K46" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-клеть</t>
+          <t>https://audius.co/Astello/neuromant-клеть</t>
         </is>
       </c>
       <c r="L46" s="12" t="n">
@@ -10528,7 +10528,7 @@
       <c r="J47" s="9" t="inlineStr"/>
       <c r="K47" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-край-бесконечно-истерзанный</t>
+          <t>https://audius.co/Astello/neuromant-край-бесконечно-истерзанный</t>
         </is>
       </c>
       <c r="L47" s="12" t="n">
@@ -10572,7 +10572,7 @@
       <c r="J48" s="9" t="inlineStr"/>
       <c r="K48" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
+          <t>https://audius.co/Astello/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
         </is>
       </c>
       <c r="L48" s="12" t="n">
@@ -10616,7 +10616,7 @@
       <c r="J49" s="9" t="inlineStr"/>
       <c r="K49" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-ненависть</t>
+          <t>https://audius.co/Astello/neuromant-ненависть</t>
         </is>
       </c>
       <c r="L49" s="12" t="n">
@@ -10664,7 +10664,7 @@
       <c r="J50" s="9" t="inlineStr"/>
       <c r="K50" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-поднимите-веки-выше</t>
+          <t>https://audius.co/Astello/neuromant-поднимите-веки-выше</t>
         </is>
       </c>
       <c r="L50" s="12" t="n">
@@ -10708,7 +10708,7 @@
       <c r="J51" s="9" t="inlineStr"/>
       <c r="K51" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-полый</t>
+          <t>https://audius.co/Astello/neuromant-полый</t>
         </is>
       </c>
       <c r="L51" s="12" t="n">
@@ -10752,7 +10752,7 @@
       <c r="J52" s="9" t="inlineStr"/>
       <c r="K52" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-последний-полет-бабочки</t>
+          <t>https://audius.co/Astello/neuromant-последний-полет-бабочки</t>
         </is>
       </c>
       <c r="L52" s="12" t="n">
@@ -10796,7 +10796,7 @@
       <c r="J53" s="9" t="inlineStr"/>
       <c r="K53" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-проклятье-крипты-darkwave</t>
+          <t>https://audius.co/Astello/neuromant-проклятье-крипты-darkwave</t>
         </is>
       </c>
       <c r="L53" s="12" t="n">
@@ -10840,7 +10840,7 @@
       <c r="J54" s="9" t="inlineStr"/>
       <c r="K54" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-проклятье-крипты</t>
+          <t>https://audius.co/Astello/neuromant-проклятье-крипты</t>
         </is>
       </c>
       <c r="L54" s="12" t="n">
@@ -10888,7 +10888,7 @@
       <c r="J55" s="9" t="inlineStr"/>
       <c r="K55" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-роксолана</t>
+          <t>https://audius.co/Astello/neuromant-роксолана</t>
         </is>
       </c>
       <c r="L55" s="12" t="n">
@@ -10932,7 +10932,7 @@
       <c r="J56" s="9" t="inlineStr"/>
       <c r="K56" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-слияние-вечности</t>
+          <t>https://audius.co/Astello/neuromant-слияние-вечности</t>
         </is>
       </c>
       <c r="L56" s="12" t="n">
@@ -10976,7 +10976,7 @@
       <c r="J57" s="9" t="inlineStr"/>
       <c r="K57" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-терон</t>
+          <t>https://audius.co/Astello/neuromant-терон</t>
         </is>
       </c>
       <c r="L57" s="12" t="n">
@@ -11020,7 +11020,7 @@
       <c r="J58" s="9" t="inlineStr"/>
       <c r="K58" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-эйдолон-1</t>
+          <t>https://audius.co/Astello/neuromant-эйдолон-1</t>
         </is>
       </c>
       <c r="L58" s="12" t="n">
@@ -11064,7 +11064,7 @@
       <c r="J59" s="9" t="inlineStr"/>
       <c r="K59" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-эйдолон-2</t>
+          <t>https://audius.co/Astello/neuromant-эйдолон-2</t>
         </is>
       </c>
       <c r="L59" s="12" t="n">
@@ -11108,7 +11108,7 @@
       <c r="J60" s="9" t="inlineStr"/>
       <c r="K60" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/neuromant-я-был-первым</t>
+          <t>https://audius.co/Astello/neuromant-я-был-первым</t>
         </is>
       </c>
       <c r="L60" s="12" t="n">
@@ -11152,7 +11152,7 @@
       <c r="J61" s="9" t="inlineStr"/>
       <c r="K61" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/nuromanta-antipod-v-0666</t>
+          <t>https://audius.co/Astello/nuromanta-antipod-v-0666</t>
         </is>
       </c>
       <c r="L61" s="12" t="n">
@@ -11192,7 +11192,7 @@
       <c r="J62" s="9" t="inlineStr"/>
       <c r="K62" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/orchestra-de-la-poh-bain-russe</t>
+          <t>https://audius.co/Astello/orchestra-de-la-poh-bain-russe</t>
         </is>
       </c>
       <c r="L62" s="12" t="n">
@@ -11232,7 +11232,7 @@
       <c r="J63" s="9" t="inlineStr"/>
       <c r="K63" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/powerwolf_ai_-_govnovoz_skysoundcc</t>
+          <t>https://audius.co/Astello/powerwolf_ai_-_govnovoz_skysoundcc</t>
         </is>
       </c>
       <c r="L63" s="12" t="n">
@@ -11272,7 +11272,7 @@
       <c r="J64" s="9" t="inlineStr"/>
       <c r="K64" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/samhain-ball</t>
+          <t>https://audius.co/Astello/samhain-ball</t>
         </is>
       </c>
       <c r="L64" s="12" t="n">
@@ -11320,7 +11320,7 @@
       <c r="J65" s="9" t="inlineStr"/>
       <c r="K65" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/teron-я-был-первым-remastered</t>
+          <t>https://audius.co/Astello/teron-я-был-первым-remastered</t>
         </is>
       </c>
       <c r="L65" s="12" t="n">
@@ -11364,7 +11364,7 @@
       <c r="J66" s="9" t="inlineStr"/>
       <c r="K66" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/trupovoz</t>
+          <t>https://audius.co/Astello/trupovoz</t>
         </is>
       </c>
       <c r="L66" s="12" t="n">
@@ -11408,7 +11408,7 @@
       <c r="J67" s="9" t="inlineStr"/>
       <c r="K67" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/vea-мое-болото</t>
+          <t>https://audius.co/Astello/vea-мое-болото</t>
         </is>
       </c>
       <c r="L67" s="12" t="n">
@@ -11452,7 +11452,7 @@
       <c r="J68" s="9" t="inlineStr"/>
       <c r="K68" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
+          <t>https://audius.co/Astello/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
         </is>
       </c>
       <c r="L68" s="12" t="n">
@@ -11496,7 +11496,7 @@
       <c r="J69" s="9" t="inlineStr"/>
       <c r="K69" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
+          <t>https://audius.co/Astello/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
         </is>
       </c>
       <c r="L69" s="12" t="n">
@@ -11540,7 +11540,7 @@
       <c r="J70" s="9" t="inlineStr"/>
       <c r="K70" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-v20</t>
+          <t>https://audius.co/Astello/warcrafter-вспоминаю-дни-v20</t>
         </is>
       </c>
       <c r="L70" s="12" t="n">
@@ -11588,7 +11588,7 @@
       <c r="J71" s="9" t="inlineStr"/>
       <c r="K71" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/альтушка-для-вия-homa-brut</t>
+          <t>https://audius.co/Astello/альтушка-для-вия-homa-brut</t>
         </is>
       </c>
       <c r="L71" s="12" t="n">
@@ -11628,7 +11628,7 @@
       <c r="J72" s="9" t="inlineStr"/>
       <c r="K72" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/бедство-элвиннского-леса</t>
+          <t>https://audius.co/Astello/бедство-элвиннского-леса</t>
         </is>
       </c>
       <c r="L72" s="12" t="n">
@@ -11668,7 +11668,7 @@
       <c r="J73" s="9" t="inlineStr"/>
       <c r="K73" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/в-склеп-древний-про́клятый-темный</t>
+          <t>https://audius.co/Astello/в-склеп-древний-про́клятый-темный</t>
         </is>
       </c>
       <c r="L73" s="12" t="n">
@@ -11712,7 +11712,7 @@
       <c r="J74" s="9" t="inlineStr"/>
       <c r="K74" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/вар-прокачка</t>
+          <t>https://audius.co/Astello/вар-прокачка</t>
         </is>
       </c>
       <c r="L74" s="12" t="n">
@@ -11752,7 +11752,7 @@
       <c r="J75" s="9" t="inlineStr"/>
       <c r="K75" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/вперед-на-брбрбрбр</t>
+          <t>https://audius.co/Astello/вперед-на-брбрбрбр</t>
         </is>
       </c>
       <c r="L75" s="12" t="n">
@@ -11792,7 +11792,7 @@
       <c r="J76" s="9" t="inlineStr"/>
       <c r="K76" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд-v3</t>
+          <t>https://audius.co/Astello/гимн-чд-v3</t>
         </is>
       </c>
       <c r="L76" s="12" t="n">
@@ -11832,7 +11832,7 @@
       <c r="J77" s="9" t="inlineStr"/>
       <c r="K77" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp</t>
+          <t>https://audius.co/Astello/гимн-чд-но-это-аниме-jp</t>
         </is>
       </c>
       <c r="L77" s="12" t="n">
@@ -11872,7 +11872,7 @@
       <c r="J78" s="9" t="inlineStr"/>
       <c r="K78" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp_metal</t>
+          <t>https://audius.co/Astello/гимн-чд-но-это-аниме-jp_metal</t>
         </is>
       </c>
       <c r="L78" s="12" t="n">
@@ -11912,7 +11912,7 @@
       <c r="J79" s="9" t="inlineStr"/>
       <c r="K79" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/гимн-чд</t>
+          <t>https://audius.co/Astello/гимн-чд</t>
         </is>
       </c>
       <c r="L79" s="12" t="n">
@@ -11952,7 +11952,7 @@
       <c r="J80" s="9" t="inlineStr"/>
       <c r="K80" s="11" t="inlineStr">
         <is>
-          <t>https://audius.co/Durachok/др-денису</t>
+          <t>https://audius.co/Astello/др-денису</t>
         </is>
       </c>
       <c r="L80" s="12" t="n">

</xml_diff>